<commit_message>
Revert "Merge branch 'Scripting' into VTB"
This reverts commit 29620843d9fdda6479231d0555d4f481241e6653, reversing
changes made to b16d38979a728e808425eeef6dcc7ac29c2efbab.
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Raising.xlsx
+++ b/Assets/StreamingAssets/Configurations/Raising.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{188BEC3A-DB4C-4F34-89CA-724DFAAF2EE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{50E5FAE0-6D8C-4C7A-945F-E71747CBD6FA}"/>
+    <workbookView windowWidth="24750" windowHeight="10480"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingEffects" sheetId="1" r:id="rId1"/>
@@ -21,9 +15,6 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -31,6 +22,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -38,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="138">
   <si>
     <t>ID</t>
   </si>
@@ -181,6 +174,27 @@
     <t>BARevenueShareRate</t>
   </si>
   <si>
+    <t>选择阶段结局</t>
+  </si>
+  <si>
+    <t>选择阶段结束</t>
+  </si>
+  <si>
+    <t>VRaisingPickPhaseEndingEffect</t>
+  </si>
+  <si>
+    <t>加遗物0</t>
+  </si>
+  <si>
+    <t>VRaisingAddRelicEffect</t>
+  </si>
+  <si>
+    <t>从卡组删除一张卡牌</t>
+  </si>
+  <si>
+    <t>VRaisingDeleteSelected</t>
+  </si>
+  <si>
     <t>Type_M</t>
   </si>
   <si>
@@ -223,6 +237,147 @@
     <t>BackGroundColor</t>
   </si>
   <si>
+    <t>DialogueNode</t>
+  </si>
+  <si>
+    <t>声乐练习</t>
+  </si>
+  <si>
+    <t>歌力+40</t>
+  </si>
+  <si>
+    <t>Practice</t>
+  </si>
+  <si>
+    <t>Stamina</t>
+  </si>
+  <si>
+    <t>#FF2160</t>
+  </si>
+  <si>
+    <t>AddSinging</t>
+  </si>
+  <si>
+    <t>游戏练习</t>
+  </si>
+  <si>
+    <t>游戏力+40</t>
+  </si>
+  <si>
+    <t>#4B58FF</t>
+  </si>
+  <si>
+    <t>AddGaming</t>
+  </si>
+  <si>
+    <t>对话练习</t>
+  </si>
+  <si>
+    <t>杂谈力+40</t>
+  </si>
+  <si>
+    <t>#FFB200</t>
+  </si>
+  <si>
+    <t>AddChatting</t>
+  </si>
+  <si>
+    <t>小憩一会</t>
+  </si>
+  <si>
+    <t>体力+25</t>
+  </si>
+  <si>
+    <t>Recovery</t>
+  </si>
+  <si>
+    <t>#00B050</t>
+  </si>
+  <si>
+    <t>Nap</t>
+  </si>
+  <si>
+    <t>外出吃饭</t>
+  </si>
+  <si>
+    <t>体力+60</t>
+  </si>
+  <si>
+    <t>Out</t>
+  </si>
+  <si>
+    <t>放一天假</t>
+  </si>
+  <si>
+    <t>体力+100</t>
+  </si>
+  <si>
+    <t>DayOff</t>
+  </si>
+  <si>
+    <t>直播成功</t>
+  </si>
+  <si>
+    <t>#00B051</t>
+  </si>
+  <si>
+    <t>StreamSuccess</t>
+  </si>
+  <si>
+    <t>直播失败</t>
+  </si>
+  <si>
+    <t>#00B052</t>
+  </si>
+  <si>
+    <t>StreamFail</t>
+  </si>
+  <si>
+    <t>昏厥</t>
+  </si>
+  <si>
+    <t>#00B053</t>
+  </si>
+  <si>
+    <t>OuttaStamina</t>
+  </si>
+  <si>
+    <t>阶段开始</t>
+  </si>
+  <si>
+    <t>#00B054</t>
+  </si>
+  <si>
+    <t>PhaseStart</t>
+  </si>
+  <si>
+    <t>阶段开始2</t>
+  </si>
+  <si>
+    <t>阶段开始3</t>
+  </si>
+  <si>
+    <t>#00B055</t>
+  </si>
+  <si>
+    <t>PhaseStart2</t>
+  </si>
+  <si>
+    <t>兼职</t>
+  </si>
+  <si>
+    <t>金钱+40</t>
+  </si>
+  <si>
+    <t>Wrok</t>
+  </si>
+  <si>
+    <t>#E5FD1F</t>
+  </si>
+  <si>
+    <t>Wrok1</t>
+  </si>
+  <si>
     <t>TurnCount</t>
   </si>
   <si>
@@ -247,9 +402,6 @@
     <t>Stream</t>
   </si>
   <si>
-    <t>Stamina</t>
-  </si>
-  <si>
     <t>#AB0580</t>
   </si>
   <si>
@@ -283,114 +435,6 @@
     <t>Ending6</t>
   </si>
   <si>
-    <t>DialogueNode</t>
-  </si>
-  <si>
-    <t>声乐练习</t>
-  </si>
-  <si>
-    <t>歌力+40</t>
-  </si>
-  <si>
-    <t>Practice</t>
-  </si>
-  <si>
-    <t>#FF2160</t>
-  </si>
-  <si>
-    <t>AddSinging</t>
-  </si>
-  <si>
-    <t>游戏练习</t>
-  </si>
-  <si>
-    <t>游戏力+40</t>
-  </si>
-  <si>
-    <t>#4B58FF</t>
-  </si>
-  <si>
-    <t>AddGaming</t>
-  </si>
-  <si>
-    <t>对话练习</t>
-  </si>
-  <si>
-    <t>杂谈力+40</t>
-  </si>
-  <si>
-    <t>#FFB200</t>
-  </si>
-  <si>
-    <t>AddChatting</t>
-  </si>
-  <si>
-    <t>小憩一会</t>
-  </si>
-  <si>
-    <t>体力+25</t>
-  </si>
-  <si>
-    <t>Recovery</t>
-  </si>
-  <si>
-    <t>#00B050</t>
-  </si>
-  <si>
-    <t>Nap</t>
-  </si>
-  <si>
-    <t>外出吃饭</t>
-  </si>
-  <si>
-    <t>体力+60</t>
-  </si>
-  <si>
-    <t>Break</t>
-  </si>
-  <si>
-    <t>放一天假</t>
-  </si>
-  <si>
-    <t>体力+100</t>
-  </si>
-  <si>
-    <t>DayOff</t>
-  </si>
-  <si>
-    <t>StreamSuccess</t>
-  </si>
-  <si>
-    <t>#00B051</t>
-  </si>
-  <si>
-    <t>StreamFail</t>
-  </si>
-  <si>
-    <t>#00B052</t>
-  </si>
-  <si>
-    <t>NoStamina</t>
-  </si>
-  <si>
-    <t>#00B053</t>
-  </si>
-  <si>
-    <t>OuttaStamina</t>
-  </si>
-  <si>
-    <t>PhaseStart</t>
-  </si>
-  <si>
-    <t>#00B054</t>
-  </si>
-  <si>
-    <t>PhaseStart2</t>
-  </si>
-  <si>
-    <t>#00B055</t>
-  </si>
-  <si>
     <t>NameOrID</t>
   </si>
   <si>
@@ -401,55 +445,172 @@
   </si>
   <si>
     <t>VPhaseEndingEventCondition</t>
-  </si>
-  <si>
-    <t>VRaisingPickPhaseEndingEffect</t>
-  </si>
-  <si>
-    <t>选择阶段结束</t>
-  </si>
-  <si>
-    <t>选择阶段结局</t>
-  </si>
-  <si>
-    <t>加遗物0</t>
-  </si>
-  <si>
-    <t>VRaisingAddRelicEffect</t>
-  </si>
-  <si>
-    <t>加遗物1</t>
-  </si>
-  <si>
-    <t>追加事件</t>
-  </si>
-  <si>
-    <t>VRaisingAddEventAfterCurrentEffect</t>
-  </si>
-  <si>
-    <t>追加事件Test</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="等线"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -486,8 +647,200 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE5FD1F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -495,11 +848,253 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -512,18 +1107,69 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  <cellStyles count="49">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="00F7BB25"/>
+      <color rgb="00E5FD1F"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -572,7 +1218,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -605,26 +1251,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -657,23 +1286,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -815,30 +1427,25 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69B7D76C-5297-47CF-900A-9659A5CEEA70}">
-  <dimension ref="A1:F24"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="3.42578125" customWidth="1"/>
-    <col min="2" max="2" width="31.42578125" customWidth="1"/>
-    <col min="3" max="3" width="29.42578125" customWidth="1"/>
-    <col min="4" max="4" width="31.7109375" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" customWidth="1"/>
-    <col min="6" max="6" width="29.5703125" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="3.425" customWidth="1"/>
+    <col min="2" max="2" width="31.425" customWidth="1"/>
+    <col min="3" max="3" width="29.425" customWidth="1"/>
+    <col min="4" max="4" width="28.425" customWidth="1"/>
+    <col min="5" max="5" width="15.2833333333333" customWidth="1"/>
+    <col min="6" max="6" width="29.5666666666667" customWidth="1"/>
+    <col min="7" max="7" width="15.7083333333333" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -858,7 +1465,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6">
       <c r="A2">
         <v>0</v>
       </c>
@@ -878,7 +1485,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6">
       <c r="A3">
         <v>1</v>
       </c>
@@ -898,7 +1505,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>2</v>
       </c>
@@ -918,7 +1525,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6">
       <c r="A5">
         <v>3</v>
       </c>
@@ -935,7 +1542,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6">
       <c r="A6">
         <v>4</v>
       </c>
@@ -952,7 +1559,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6">
       <c r="A7">
         <v>5</v>
       </c>
@@ -969,7 +1576,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4">
       <c r="A8">
         <v>6</v>
       </c>
@@ -983,7 +1590,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4">
       <c r="A9">
         <v>7</v>
       </c>
@@ -997,7 +1604,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5">
       <c r="A10">
         <v>8</v>
       </c>
@@ -1014,7 +1621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6">
       <c r="A11">
         <v>9</v>
       </c>
@@ -1031,7 +1638,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6">
       <c r="A12">
         <v>10</v>
       </c>
@@ -1048,7 +1655,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6">
       <c r="A13">
         <v>11</v>
       </c>
@@ -1065,7 +1672,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6">
       <c r="A14">
         <v>12</v>
       </c>
@@ -1082,7 +1689,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6">
       <c r="A15">
         <v>13</v>
       </c>
@@ -1099,7 +1706,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6">
       <c r="A16">
         <v>14</v>
       </c>
@@ -1116,7 +1723,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6">
       <c r="A17">
         <v>15</v>
       </c>
@@ -1133,7 +1740,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6">
       <c r="A18">
         <v>16</v>
       </c>
@@ -1150,7 +1757,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6">
       <c r="A19">
         <v>17</v>
       </c>
@@ -1167,7 +1774,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6">
       <c r="A20">
         <v>18</v>
       </c>
@@ -1184,90 +1791,71 @@
         <v>46</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4">
       <c r="A21">
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>123</v>
+        <v>47</v>
       </c>
       <c r="C21" t="s">
-        <v>122</v>
+        <v>48</v>
       </c>
       <c r="D21" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
       <c r="A22">
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>124</v>
+        <v>50</v>
       </c>
       <c r="C22" t="s">
-        <v>124</v>
+        <v>50</v>
       </c>
       <c r="D22" t="s">
-        <v>125</v>
+        <v>51</v>
       </c>
       <c r="F22">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4">
       <c r="A23">
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>126</v>
+        <v>52</v>
       </c>
       <c r="C23" t="s">
-        <v>126</v>
+        <v>52</v>
       </c>
       <c r="D23" t="s">
-        <v>125</v>
-      </c>
-      <c r="F23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>22</v>
-      </c>
-      <c r="B24" t="s">
-        <v>129</v>
-      </c>
-      <c r="C24" t="s">
-        <v>127</v>
-      </c>
-      <c r="D24" t="s">
-        <v>128</v>
-      </c>
-      <c r="F24" t="s">
-        <v>84</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C731E613-AE8E-4BCD-9551-0D399E493DD1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="3" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="17.28515625" customWidth="1"/>
-    <col min="4" max="4" width="20.140625" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="17.2833333333333" customWidth="1"/>
+    <col min="4" max="4" width="20.1416666666667" customWidth="1"/>
+    <col min="5" max="5" width="19.7083333333333" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1284,74 +1872,76 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="C2" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="D2" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="E2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="E3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="E4" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2983CD5-09FC-448D-B584-53935FACCACB}">
-  <dimension ref="A1:J12"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:J13"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" customWidth="1"/>
-    <col min="2" max="2" width="23.28515625" customWidth="1"/>
-    <col min="3" max="3" width="20.140625" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" customWidth="1"/>
-    <col min="5" max="5" width="8.140625" customWidth="1"/>
-    <col min="6" max="6" width="8.42578125" customWidth="1"/>
-    <col min="7" max="7" width="6.85546875" customWidth="1"/>
-    <col min="8" max="8" width="10.28515625" customWidth="1"/>
-    <col min="9" max="9" width="15.5703125" customWidth="1"/>
-    <col min="10" max="10" width="16.85546875" customWidth="1"/>
+    <col min="1" max="1" width="10.425" customWidth="1"/>
+    <col min="2" max="2" width="23.2833333333333" customWidth="1"/>
+    <col min="3" max="3" width="20.1416666666667" customWidth="1"/>
+    <col min="4" max="4" width="10.1416666666667" customWidth="1"/>
+    <col min="5" max="5" width="8.14166666666667" customWidth="1"/>
+    <col min="6" max="6" width="8.425" customWidth="1"/>
+    <col min="7" max="7" width="6.85833333333333" customWidth="1"/>
+    <col min="8" max="8" width="10.2833333333333" customWidth="1"/>
+    <col min="9" max="9" width="15.5666666666667" customWidth="1"/>
+    <col min="10" max="10" width="16.8583333333333" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1365,387 +1955,436 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="F1" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="G1" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="H1" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="I1" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="J1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="D2" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G2">
         <v>10</v>
       </c>
       <c r="H2" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="J2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="C3" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="D3" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="E3">
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G3">
         <v>10</v>
       </c>
       <c r="H3" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="J3" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="C4" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="D4" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G4">
         <v>10</v>
       </c>
       <c r="H4" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="J4" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="C5" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="D5" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="J5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="C6" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D6" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="E6">
         <v>2</v>
       </c>
       <c r="F6" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="J6" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="D7" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="E7">
         <v>3</v>
       </c>
       <c r="F7" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="J7" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>106</v>
+        <v>94</v>
+      </c>
+      <c r="C8" t="s">
+        <v>94</v>
       </c>
       <c r="D8" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="E8">
         <v>0</v>
       </c>
       <c r="F8" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G8">
         <v>0</v>
       </c>
       <c r="H8" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="J8" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>108</v>
+        <v>97</v>
+      </c>
+      <c r="C9" t="s">
+        <v>97</v>
       </c>
       <c r="D9" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="E9">
         <v>0</v>
       </c>
       <c r="F9" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G9">
         <v>0</v>
       </c>
       <c r="H9" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="J9" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
       <c r="A10">
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>110</v>
+        <v>100</v>
+      </c>
+      <c r="C10" t="s">
+        <v>100</v>
       </c>
       <c r="D10" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="E10">
         <v>0</v>
       </c>
       <c r="F10" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G10">
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="J10" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
       <c r="A11">
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>113</v>
+        <v>103</v>
+      </c>
+      <c r="C11" t="s">
+        <v>103</v>
       </c>
       <c r="D11" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="E11">
         <v>0</v>
       </c>
       <c r="F11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G11">
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="J11" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
       <c r="A12">
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>115</v>
+        <v>106</v>
+      </c>
+      <c r="C12" t="s">
+        <v>107</v>
       </c>
       <c r="D12" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="E12">
         <v>0</v>
       </c>
       <c r="F12" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G12">
         <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="J12" t="s">
-        <v>115</v>
+        <v>109</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>110</v>
+      </c>
+      <c r="C13" t="s">
+        <v>111</v>
+      </c>
+      <c r="D13" t="s">
+        <v>112</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13" t="s">
+        <v>72</v>
+      </c>
+      <c r="G13">
+        <v>10</v>
+      </c>
+      <c r="H13" t="s">
+        <v>85</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="J13" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64D15A77-1535-49E5-8565-BF3C734F79F3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:O10"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="8.42578125" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" customWidth="1"/>
-    <col min="3" max="3" width="22.28515625" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" customWidth="1"/>
-    <col min="5" max="6" width="11.42578125" customWidth="1"/>
-    <col min="7" max="7" width="6.7109375" customWidth="1"/>
-    <col min="9" max="9" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="8.425" customWidth="1"/>
+    <col min="2" max="2" width="21.8583333333333" customWidth="1"/>
+    <col min="3" max="3" width="22.2833333333333" customWidth="1"/>
+    <col min="4" max="4" width="11.5666666666667" customWidth="1"/>
+    <col min="5" max="6" width="11.425" customWidth="1"/>
+    <col min="7" max="7" width="6.70833333333333" customWidth="1"/>
+    <col min="9" max="9" width="15.7083333333333" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="10.85546875" customWidth="1"/>
-    <col min="12" max="12" width="15.85546875" customWidth="1"/>
-    <col min="13" max="13" width="13.140625" customWidth="1"/>
-    <col min="14" max="14" width="10.42578125" customWidth="1"/>
-    <col min="15" max="15" width="12.7109375" customWidth="1"/>
+    <col min="11" max="11" width="10.8583333333333" customWidth="1"/>
+    <col min="12" max="12" width="15.8583333333333" customWidth="1"/>
+    <col min="13" max="13" width="13.1416666666667" customWidth="1"/>
+    <col min="14" max="14" width="10.425" customWidth="1"/>
+    <col min="15" max="15" width="12.7083333333333" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1759,66 +2398,66 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="F1" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="G1" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="H1" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="I1" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="J1" t="s">
-        <v>61</v>
+        <v>115</v>
       </c>
       <c r="K1" t="s">
-        <v>62</v>
+        <v>116</v>
       </c>
       <c r="L1" t="s">
-        <v>63</v>
+        <v>117</v>
       </c>
       <c r="M1" t="s">
-        <v>64</v>
+        <v>118</v>
       </c>
       <c r="N1" t="s">
-        <v>65</v>
+        <v>119</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>121</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>121</v>
       </c>
       <c r="D2" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G2">
         <v>25</v>
       </c>
       <c r="H2" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>70</v>
+        <v>123</v>
       </c>
       <c r="J2">
         <v>3</v>
@@ -1836,33 +2475,33 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>124</v>
       </c>
       <c r="C3" t="s">
-        <v>71</v>
+        <v>124</v>
       </c>
       <c r="D3" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="E3">
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G3">
         <v>25</v>
       </c>
       <c r="H3" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>70</v>
+        <v>123</v>
       </c>
       <c r="J3">
         <v>5</v>
@@ -1880,33 +2519,33 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>72</v>
+        <v>125</v>
       </c>
       <c r="C4" t="s">
-        <v>72</v>
+        <v>125</v>
       </c>
       <c r="D4" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G4">
         <v>25</v>
       </c>
       <c r="H4" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>70</v>
+        <v>123</v>
       </c>
       <c r="J4">
         <v>10</v>
@@ -1924,33 +2563,33 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>73</v>
+        <v>126</v>
       </c>
       <c r="C5" t="s">
-        <v>74</v>
+        <v>127</v>
       </c>
       <c r="D5" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="E5">
         <v>3</v>
       </c>
       <c r="F5" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>70</v>
+        <v>123</v>
       </c>
       <c r="J5">
         <v>10</v>
@@ -1971,33 +2610,33 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>75</v>
+        <v>128</v>
       </c>
       <c r="C6" t="s">
-        <v>74</v>
+        <v>127</v>
       </c>
       <c r="D6" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="E6">
         <v>3</v>
       </c>
       <c r="F6" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>70</v>
+        <v>123</v>
       </c>
       <c r="J6">
         <v>10</v>
@@ -2015,36 +2654,36 @@
         <v>7</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>77</v>
+        <v>130</v>
       </c>
       <c r="C7" t="s">
-        <v>74</v>
+        <v>127</v>
       </c>
       <c r="D7" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="E7">
         <v>3</v>
       </c>
       <c r="F7" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>70</v>
+        <v>123</v>
       </c>
       <c r="J7">
         <v>10</v>
@@ -2065,33 +2704,33 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>78</v>
+        <v>131</v>
       </c>
       <c r="C8" t="s">
-        <v>74</v>
+        <v>127</v>
       </c>
       <c r="D8" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="E8">
         <v>3</v>
       </c>
       <c r="F8" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G8">
         <v>0</v>
       </c>
       <c r="H8" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>70</v>
+        <v>123</v>
       </c>
       <c r="J8">
         <v>10</v>
@@ -2112,33 +2751,33 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>79</v>
+        <v>132</v>
       </c>
       <c r="C9" t="s">
-        <v>74</v>
+        <v>127</v>
       </c>
       <c r="D9" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="E9">
         <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G9">
         <v>0</v>
       </c>
       <c r="H9" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>70</v>
+        <v>123</v>
       </c>
       <c r="J9">
         <v>10</v>
@@ -2156,36 +2795,36 @@
         <v>7</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
       <c r="A10">
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>80</v>
+        <v>133</v>
       </c>
       <c r="C10" t="s">
-        <v>74</v>
+        <v>127</v>
       </c>
       <c r="D10" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="E10">
         <v>3</v>
       </c>
       <c r="F10" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G10">
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>70</v>
+        <v>123</v>
       </c>
       <c r="J10">
         <v>10</v>
@@ -2208,23 +2847,25 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4476F971-FB5B-4F8B-812B-3D6B61D9FDFF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="3" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" customWidth="1"/>
-    <col min="2" max="2" width="19.42578125" customWidth="1"/>
-    <col min="3" max="3" width="22.85546875" customWidth="1"/>
-    <col min="4" max="4" width="31.140625" customWidth="1"/>
-    <col min="5" max="5" width="23.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.5666666666667" customWidth="1"/>
+    <col min="2" max="2" width="19.425" customWidth="1"/>
+    <col min="3" max="3" width="22.8583333333333" customWidth="1"/>
+    <col min="4" max="4" width="31.1416666666667" customWidth="1"/>
+    <col min="5" max="5" width="23.425" customWidth="1"/>
+    <col min="6" max="6" width="9.70833333333333" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2238,13 +2879,13 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="F1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2">
         <v>0</v>
       </c>
@@ -2255,7 +2896,7 @@
         <v>36</v>
       </c>
       <c r="D2" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="E2" t="s">
         <v>8</v>
@@ -2264,7 +2905,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2275,7 +2916,7 @@
         <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="E3" t="s">
         <v>8</v>
@@ -2284,7 +2925,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2295,16 +2936,17 @@
         <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
       <c r="E4">
         <v>5</v>
       </c>
       <c r="F4" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
FIXED VRaisingDeleteSelected NOT FOUND
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Raising.xlsx
+++ b/Assets/StreamingAssets/Configurations/Raising.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53EEAC22-65F8-4F45-A118-8F8C7376CE54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE3788F3-7A84-431A-A68D-41880868EA7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{50E5FAE0-6D8C-4C7A-945F-E71747CBD6FA}"/>
+    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{50E5FAE0-6D8C-4C7A-945F-E71747CBD6FA}"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingEffects" sheetId="1" r:id="rId1"/>
@@ -839,7 +839,7 @@
     <col min="2" max="2" width="31.42578125" customWidth="1"/>
     <col min="3" max="3" width="29.42578125" customWidth="1"/>
     <col min="4" max="4" width="31.7109375" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" customWidth="1"/>
+    <col min="5" max="5" width="11.42578125" customWidth="1"/>
     <col min="6" max="6" width="29.5703125" customWidth="1"/>
     <col min="7" max="7" width="15.7109375" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
added coop upgrade event
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Raising.xlsx
+++ b/Assets/StreamingAssets/Configurations/Raising.xlsx
@@ -1,18 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EC90EF8-8192-465A-B5AC-1877F2A0AEBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="10480"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingEffects" sheetId="1" r:id="rId1"/>
     <sheet name="CardConditions" sheetId="2" r:id="rId2"/>
     <sheet name="DialogueEvents" sheetId="4" r:id="rId3"/>
     <sheet name="StreamEvents" sheetId="3" r:id="rId4"/>
-    <sheet name="PhaseEndingConditions" sheetId="5" r:id="rId5"/>
-    <sheet name="PlacingConditions" sheetId="6" r:id="rId6"/>
+    <sheet name="PlacingConditions" sheetId="6" r:id="rId5"/>
+    <sheet name="PhaseEndingConditions" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -23,8 +29,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -32,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="176">
   <si>
     <t>ID</t>
   </si>
@@ -514,18 +518,6 @@
     <t>杂谈回成功事件</t>
   </si>
   <si>
-    <t>进阶唱歌练习</t>
-  </si>
-  <si>
-    <t>歌力+60</t>
-  </si>
-  <si>
-    <t>进阶游戏练习</t>
-  </si>
-  <si>
-    <t>进阶杂谈练习</t>
-  </si>
-  <si>
     <t>TurnCount</t>
   </si>
   <si>
@@ -602,23 +594,47 @@
   </si>
   <si>
     <t xml:space="preserve"> TargetValue</t>
+  </si>
+  <si>
+    <t>VAttributePlacingCondition</t>
+  </si>
+  <si>
+    <t>CASingingAbility,200</t>
+  </si>
+  <si>
+    <t>VTimeOfDayPlacingCondition</t>
+  </si>
+  <si>
+    <t>VDayPlacingCondition</t>
+  </si>
+  <si>
+    <t>add coop level for goomba</t>
+  </si>
+  <si>
+    <t>VRaisingAddCoopValueEffect</t>
+  </si>
+  <si>
+    <t>UPGRADE level for goomba</t>
+  </si>
+  <si>
+    <t>VRaisingUpgradeCoopLevel</t>
+  </si>
+  <si>
+    <t>Upgrade Level for goomba</t>
+  </si>
+  <si>
+    <t>GoombaUpgradelv1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="22">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -629,157 +645,19 @@
       <charset val="134"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="10.5"/>
       <color theme="1"/>
       <name val="Consolas"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="40">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -828,194 +706,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1023,251 +715,9 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1306,66 +756,22 @@
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="000BF30B"/>
+      <color rgb="FF0BF30B"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1623,22 +1029,22 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F28"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.425" customWidth="1"/>
-    <col min="2" max="2" width="31.425" customWidth="1"/>
-    <col min="3" max="3" width="29.425" customWidth="1"/>
-    <col min="4" max="4" width="31.7083333333333" customWidth="1"/>
-    <col min="5" max="5" width="15.2833333333333" customWidth="1"/>
-    <col min="6" max="6" width="29.5666666666667" customWidth="1"/>
-    <col min="7" max="7" width="15.7083333333333" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="31.42578125" customWidth="1"/>
+    <col min="3" max="3" width="29.42578125" customWidth="1"/>
+    <col min="4" max="4" width="31.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" customWidth="1"/>
+    <col min="6" max="6" width="29.5703125" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1772,7 +1178,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:6">
       <c r="A8">
         <v>6</v>
       </c>
@@ -1786,7 +1192,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:6">
       <c r="A9">
         <v>7</v>
       </c>
@@ -1800,7 +1206,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:6">
       <c r="A10">
         <v>8</v>
       </c>
@@ -1987,7 +1393,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:6">
       <c r="A21">
         <v>19</v>
       </c>
@@ -2052,7 +1458,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:6">
       <c r="A25">
         <v>23</v>
       </c>
@@ -2066,7 +1472,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:6">
       <c r="A26">
         <v>24</v>
       </c>
@@ -2083,23 +1489,52 @@
         <v>3</v>
       </c>
     </row>
+    <row r="27" spans="1:6">
+      <c r="A27">
+        <v>25</v>
+      </c>
+      <c r="B27" t="s">
+        <v>170</v>
+      </c>
+      <c r="C27" t="s">
+        <v>170</v>
+      </c>
+      <c r="D27" t="s">
+        <v>171</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28">
+        <v>26</v>
+      </c>
+      <c r="B28" t="s">
+        <v>172</v>
+      </c>
+      <c r="D28" t="s">
+        <v>173</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="7" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="17.2833333333333" customWidth="1"/>
-    <col min="4" max="4" width="20.1416666666667" customWidth="1"/>
-    <col min="5" max="5" width="19.7083333333333" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" customWidth="1"/>
+    <col min="5" max="5" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2219,30 +1654,28 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:K21"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="10.425" style="3" customWidth="1"/>
-    <col min="2" max="2" width="23.2833333333333" style="3" customWidth="1"/>
-    <col min="3" max="3" width="27.7083333333333" style="3" customWidth="1"/>
-    <col min="4" max="4" width="10.1416666666667" style="3" customWidth="1"/>
-    <col min="5" max="5" width="8.14166666666667" style="3" customWidth="1"/>
-    <col min="6" max="6" width="8.425" style="3" customWidth="1"/>
-    <col min="7" max="7" width="6.85833333333333" style="3" customWidth="1"/>
-    <col min="8" max="8" width="10.2833333333333" style="3" customWidth="1"/>
-    <col min="9" max="9" width="15.5666666666667" style="3" customWidth="1"/>
-    <col min="10" max="11" width="16.8583333333333" style="3" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" style="3" customWidth="1"/>
+    <col min="7" max="7" width="6.85546875" style="3" customWidth="1"/>
+    <col min="8" max="8" width="10.28515625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" style="3" customWidth="1"/>
+    <col min="10" max="11" width="16.85546875" style="3" customWidth="1"/>
     <col min="12" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:11">
+    <row r="1" spans="1:11" ht="30" customHeight="1">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2277,7 +1710,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="2" customHeight="1" spans="1:11">
+    <row r="2" spans="1:11" ht="30" customHeight="1">
       <c r="A2" s="3">
         <v>0</v>
       </c>
@@ -2309,7 +1742,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="3" customHeight="1" spans="1:11">
+    <row r="3" spans="1:11" ht="30" customHeight="1">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -2341,7 +1774,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="4" customHeight="1" spans="1:11">
+    <row r="4" spans="1:11" ht="30" customHeight="1">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -2373,7 +1806,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="5" customHeight="1" spans="1:11">
+    <row r="5" spans="1:11" ht="30" customHeight="1">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -2405,7 +1838,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1" spans="1:11">
+    <row r="6" spans="1:11" ht="48" customHeight="1">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -2437,7 +1870,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="7" customHeight="1" spans="1:11">
+    <row r="7" spans="1:11" ht="30" customHeight="1">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -2469,7 +1902,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="8" customHeight="1" spans="1:11">
+    <row r="8" spans="1:11" ht="30" customHeight="1">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -2501,7 +1934,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="9" customHeight="1" spans="1:11">
+    <row r="9" spans="1:11" ht="30" customHeight="1">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -2533,7 +1966,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="10" customHeight="1" spans="1:11">
+    <row r="10" spans="1:11" ht="30" customHeight="1">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -2565,7 +1998,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="11" customHeight="1" spans="1:11">
+    <row r="11" spans="1:11" ht="30" customHeight="1">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -2597,7 +2030,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="12" customHeight="1" spans="1:11">
+    <row r="12" spans="1:11" ht="30" customHeight="1">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -2629,7 +2062,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="13" customHeight="1" spans="1:11">
+    <row r="13" spans="1:11" ht="30" customHeight="1">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -2661,7 +2094,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="14" customHeight="1" spans="1:11">
+    <row r="14" spans="1:11" ht="30" customHeight="1">
       <c r="A14" s="3">
         <v>12</v>
       </c>
@@ -2693,7 +2126,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="15" customHeight="1" spans="1:9">
+    <row r="15" spans="1:11" ht="30" customHeight="1">
       <c r="A15" s="3">
         <v>13</v>
       </c>
@@ -2722,7 +2155,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="16" customHeight="1" spans="1:11">
+    <row r="16" spans="1:11" ht="30" customHeight="1">
       <c r="A16" s="3">
         <v>14</v>
       </c>
@@ -2754,7 +2187,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="17" customHeight="1" spans="1:11">
+    <row r="17" spans="1:11" ht="30" customHeight="1">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -2786,7 +2219,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="18" customHeight="1" spans="1:11">
+    <row r="18" spans="1:11" ht="30" customHeight="1">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -2818,59 +2251,60 @@
         <v>136</v>
       </c>
     </row>
-    <row r="19" customHeight="1" spans="1:3">
+    <row r="19" spans="1:11" ht="30" customHeight="1">
       <c r="A19" s="3">
         <v>17</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="20" customHeight="1" spans="1:2">
-      <c r="A20" s="3">
-        <v>18</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="21" customHeight="1" spans="1:2">
-      <c r="A21" s="3">
-        <v>19</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>143</v>
+        <v>174</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E19" s="3">
+        <v>1</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="G19" s="3">
+        <v>0</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="I19" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>175</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:P10"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.425" customWidth="1"/>
-    <col min="2" max="2" width="21.8583333333333" customWidth="1"/>
-    <col min="3" max="3" width="22.2833333333333" customWidth="1"/>
-    <col min="4" max="4" width="11.5666666666667" customWidth="1"/>
-    <col min="5" max="6" width="11.425" customWidth="1"/>
-    <col min="7" max="7" width="6.70833333333333" customWidth="1"/>
-    <col min="9" max="9" width="15.7083333333333" customWidth="1"/>
-    <col min="10" max="10" width="16.3333333333333" customWidth="1"/>
+    <col min="1" max="1" width="8.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" customWidth="1"/>
+    <col min="3" max="3" width="22.28515625" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" customWidth="1"/>
+    <col min="5" max="6" width="11.42578125" customWidth="1"/>
+    <col min="7" max="7" width="6.7109375" customWidth="1"/>
+    <col min="9" max="9" width="15.7109375" customWidth="1"/>
+    <col min="10" max="10" width="15.140625" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="10.8583333333333" customWidth="1"/>
-    <col min="13" max="13" width="15.8583333333333" customWidth="1"/>
-    <col min="14" max="14" width="13.1416666666667" customWidth="1"/>
-    <col min="15" max="15" width="10.425" customWidth="1"/>
-    <col min="16" max="16" width="12.7083333333333" customWidth="1"/>
+    <col min="12" max="12" width="10.85546875" customWidth="1"/>
+    <col min="13" max="13" width="15.85546875" customWidth="1"/>
+    <col min="14" max="14" width="13.140625" customWidth="1"/>
+    <col min="15" max="15" width="10.42578125" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -2905,36 +2339,36 @@
         <v>81</v>
       </c>
       <c r="K1" t="s">
+        <v>140</v>
+      </c>
+      <c r="L1" t="s">
+        <v>141</v>
+      </c>
+      <c r="M1" t="s">
+        <v>142</v>
+      </c>
+      <c r="N1" t="s">
+        <v>143</v>
+      </c>
+      <c r="O1" t="s">
         <v>144</v>
       </c>
-      <c r="L1" t="s">
+      <c r="P1" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M1" t="s">
+    </row>
+    <row r="2" spans="1:16">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
         <v>146</v>
       </c>
-      <c r="N1" t="s">
+      <c r="C2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D2" t="s">
         <v>147</v>
-      </c>
-      <c r="O1" t="s">
-        <v>148</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C2" t="s">
-        <v>150</v>
-      </c>
-      <c r="D2" t="s">
-        <v>151</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2946,10 +2380,13 @@
         <v>25</v>
       </c>
       <c r="H2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
+      </c>
+      <c r="J2" t="s">
+        <v>72</v>
       </c>
       <c r="K2">
         <v>8</v>
@@ -2967,18 +2404,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:16">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C3" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="D3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2990,10 +2427,10 @@
         <v>25</v>
       </c>
       <c r="H3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="K3">
         <v>8</v>
@@ -3011,18 +2448,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:16">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C4" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D4" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -3034,10 +2471,10 @@
         <v>25</v>
       </c>
       <c r="H4" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="K4">
         <v>8</v>
@@ -3060,16 +2497,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C5" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D5" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" t="s">
         <v>85</v>
@@ -3078,10 +2515,10 @@
         <v>40</v>
       </c>
       <c r="H5" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="K5">
         <v>10</v>
@@ -3107,13 +2544,13 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C6" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D6" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E6">
         <v>3</v>
@@ -3125,10 +2562,10 @@
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="K6">
         <v>10</v>
@@ -3146,7 +2583,7 @@
         <v>7</v>
       </c>
       <c r="P6" s="4" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:16">
@@ -3154,13 +2591,13 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C7" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D7" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E7">
         <v>3</v>
@@ -3172,10 +2609,10 @@
         <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="K7">
         <v>10</v>
@@ -3201,13 +2638,13 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C8" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D8" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E8">
         <v>3</v>
@@ -3219,10 +2656,10 @@
         <v>0</v>
       </c>
       <c r="H8" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="K8">
         <v>10</v>
@@ -3248,13 +2685,13 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C9" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D9" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E9">
         <v>3</v>
@@ -3266,10 +2703,10 @@
         <v>0</v>
       </c>
       <c r="H9" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="K9">
         <v>10</v>
@@ -3287,7 +2724,7 @@
         <v>7</v>
       </c>
       <c r="P9" s="4" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -3295,13 +2732,13 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C10" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D10" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E10">
         <v>3</v>
@@ -3313,10 +2750,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="K10">
         <v>10</v>
@@ -3339,22 +2776,87 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="3.140625" customWidth="1"/>
+    <col min="2" max="2" width="6.7109375" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" customWidth="1"/>
+    <col min="4" max="4" width="26.5703125" customWidth="1"/>
+    <col min="5" max="5" width="19.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>164</v>
+      </c>
+      <c r="E1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
+        <v>166</v>
+      </c>
+      <c r="E2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>168</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="3" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.5666666666667" customWidth="1"/>
-    <col min="2" max="2" width="19.425" customWidth="1"/>
-    <col min="3" max="3" width="22.8583333333333" customWidth="1"/>
-    <col min="4" max="4" width="31.1416666666667" customWidth="1"/>
-    <col min="5" max="5" width="23.425" customWidth="1"/>
-    <col min="6" max="6" width="9.70833333333333" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" customWidth="1"/>
+    <col min="3" max="3" width="22.85546875" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -3371,10 +2873,10 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="F1" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -3388,7 +2890,7 @@
         <v>36</v>
       </c>
       <c r="D2" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="E2" t="s">
         <v>8</v>
@@ -3408,7 +2910,7 @@
         <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="E3" t="s">
         <v>8</v>
@@ -3428,7 +2930,7 @@
         <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E4">
         <v>5</v>
@@ -3439,42 +2941,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultColWidth="8.66666666666667" defaultRowHeight="14" outlineLevelCol="4"/>
-  <cols>
-    <col min="1" max="1" width="3.08333333333333" customWidth="1"/>
-    <col min="2" max="2" width="6.66666666666667" customWidth="1"/>
-    <col min="3" max="3" width="10.4166666666667" customWidth="1"/>
-    <col min="4" max="4" width="5.66666666666667" customWidth="1"/>
-    <col min="5" max="5" width="11.4166666666667" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>167</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>168</v>
-      </c>
-      <c r="E1" t="s">
-        <v>169</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ADDED BASE COOP EVENT
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Raising.xlsx
+++ b/Assets/StreamingAssets/Configurations/Raising.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5ABEAC9-B725-45BB-9E39-457E99B35C94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A61D548-D8F1-4F0A-B678-F410AEB27FFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingEffects" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="207">
   <si>
     <t>ID</t>
   </si>
@@ -1612,6 +1612,12 @@
       <c r="B28" t="s">
         <v>63</v>
       </c>
+      <c r="C28" t="s">
+        <v>61</v>
+      </c>
+      <c r="D28" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29">
@@ -1620,6 +1626,12 @@
       <c r="B29" t="s">
         <v>64</v>
       </c>
+      <c r="C29" t="s">
+        <v>61</v>
+      </c>
+      <c r="D29" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30">
@@ -1628,6 +1640,12 @@
       <c r="B30" t="s">
         <v>65</v>
       </c>
+      <c r="C30" t="s">
+        <v>61</v>
+      </c>
+      <c r="D30" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31">
@@ -1635,6 +1653,12 @@
       </c>
       <c r="B31" t="s">
         <v>66</v>
+      </c>
+      <c r="C31" t="s">
+        <v>61</v>
+      </c>
+      <c r="D31" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -2644,7 +2668,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.42578125" customWidth="1"/>
@@ -3200,6 +3224,12 @@
       <c r="M12">
         <v>80</v>
       </c>
+      <c r="N12">
+        <v>6</v>
+      </c>
+      <c r="O12">
+        <v>7</v>
+      </c>
     </row>
     <row r="13" spans="1:16">
       <c r="A13">
@@ -3238,10 +3268,11 @@
       <c r="M13">
         <v>80</v>
       </c>
-    </row>
-    <row r="14" spans="1:16">
-      <c r="A14">
-        <v>12</v>
+      <c r="N13">
+        <v>6</v>
+      </c>
+      <c r="O13">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added account system and a new effect
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Raising.xlsx
+++ b/Assets/StreamingAssets/Configurations/Raising.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54FCF125-C83C-492F-9E96-93243EAE0330}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="22190" windowHeight="9040" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingEffects" sheetId="1" r:id="rId1"/>
@@ -25,8 +31,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -916,18 +920,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="22">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -938,157 +936,13 @@
       <charset val="134"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="10.5"/>
       <color theme="1"/>
       <name val="Consolas"/>
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="41">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1121,7 +975,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.0999786370433668"/>
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1143,194 +997,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1338,251 +1006,9 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1626,70 +1052,26 @@
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="000BF30B"/>
-      <color rgb="00E3A7F7"/>
-      <color rgb="00F567ED"/>
-      <color rgb="00DEBA2C"/>
-      <color rgb="00FD460D"/>
+      <color rgb="FF0BF30B"/>
+      <color rgb="FFE3A7F7"/>
+      <color rgb="FFF567ED"/>
+      <color rgb="FFDEBA2C"/>
+      <color rgb="FFFD460D"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1947,22 +1329,22 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F43"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.425" customWidth="1"/>
-    <col min="2" max="2" width="31.425" customWidth="1"/>
-    <col min="3" max="3" width="29.425" customWidth="1"/>
-    <col min="4" max="4" width="31.7083333333333" customWidth="1"/>
-    <col min="5" max="5" width="15.2833333333333" customWidth="1"/>
-    <col min="6" max="6" width="29.5666666666667" customWidth="1"/>
-    <col min="7" max="7" width="15.7083333333333" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="31.42578125" customWidth="1"/>
+    <col min="3" max="3" width="29.42578125" customWidth="1"/>
+    <col min="4" max="4" width="31.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" customWidth="1"/>
+    <col min="6" max="6" width="29.5703125" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -2096,7 +1478,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:6">
       <c r="A8">
         <v>6</v>
       </c>
@@ -2110,7 +1492,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:6">
       <c r="A9">
         <v>7</v>
       </c>
@@ -2124,7 +1506,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:6">
       <c r="A10">
         <v>8</v>
       </c>
@@ -2152,7 +1534,7 @@
         <v>14</v>
       </c>
       <c r="F11" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2169,7 +1551,7 @@
         <v>14</v>
       </c>
       <c r="F12" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2186,7 +1568,7 @@
         <v>14</v>
       </c>
       <c r="F13" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2203,7 +1585,7 @@
         <v>14</v>
       </c>
       <c r="F14" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -2220,7 +1602,7 @@
         <v>14</v>
       </c>
       <c r="F15" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2237,7 +1619,7 @@
         <v>14</v>
       </c>
       <c r="F16" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -2308,7 +1690,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:6">
       <c r="A21">
         <v>19</v>
       </c>
@@ -2373,7 +1755,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:6">
       <c r="A25">
         <v>23</v>
       </c>
@@ -2407,7 +1789,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:6">
       <c r="A27">
         <v>25</v>
       </c>
@@ -2602,7 +1984,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:6">
       <c r="A39">
         <v>37</v>
       </c>
@@ -2677,35 +2059,33 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:W27"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.425" customWidth="1"/>
-    <col min="2" max="2" width="21.8583333333333" customWidth="1"/>
-    <col min="3" max="3" width="22.2833333333333" customWidth="1"/>
-    <col min="4" max="4" width="11.5666666666667" customWidth="1"/>
-    <col min="5" max="6" width="11.425" customWidth="1"/>
-    <col min="7" max="7" width="6.70833333333333" customWidth="1"/>
-    <col min="9" max="9" width="8.14166666666667" customWidth="1"/>
-    <col min="10" max="10" width="15.425" customWidth="1"/>
-    <col min="11" max="11" width="10.7083333333333" customWidth="1"/>
-    <col min="12" max="12" width="3.28333333333333" customWidth="1"/>
-    <col min="13" max="13" width="6.425" customWidth="1"/>
-    <col min="14" max="14" width="11.7083333333333" customWidth="1"/>
-    <col min="15" max="15" width="10.2833333333333" customWidth="1"/>
-    <col min="16" max="16" width="10.7083333333333" customWidth="1"/>
-    <col min="17" max="17" width="11.8583333333333" customWidth="1"/>
-    <col min="18" max="18" width="8.28333333333333" customWidth="1"/>
-    <col min="19" max="19" width="10.1416666666667" customWidth="1"/>
-    <col min="20" max="20" width="14.1416666666667" customWidth="1"/>
-    <col min="21" max="21" width="10.2833333333333" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" customWidth="1"/>
+    <col min="3" max="3" width="22.28515625" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" customWidth="1"/>
+    <col min="5" max="6" width="11.42578125" customWidth="1"/>
+    <col min="7" max="7" width="6.7109375" customWidth="1"/>
+    <col min="9" max="9" width="8.140625" customWidth="1"/>
+    <col min="10" max="10" width="15.42578125" customWidth="1"/>
+    <col min="11" max="11" width="10.7109375" customWidth="1"/>
+    <col min="12" max="12" width="3.28515625" customWidth="1"/>
+    <col min="13" max="13" width="6.42578125" customWidth="1"/>
+    <col min="14" max="14" width="11.7109375" customWidth="1"/>
+    <col min="15" max="15" width="10.28515625" customWidth="1"/>
+    <col min="16" max="16" width="10.7109375" customWidth="1"/>
+    <col min="17" max="17" width="11.85546875" customWidth="1"/>
+    <col min="18" max="18" width="8.28515625" customWidth="1"/>
+    <col min="19" max="19" width="10.140625" customWidth="1"/>
+    <col min="20" max="20" width="14.140625" customWidth="1"/>
+    <col min="21" max="21" width="10.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -2779,7 +2159,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="2" spans="1:20">
+    <row r="2" spans="1:23">
       <c r="A2">
         <v>0</v>
       </c>
@@ -2838,7 +2218,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:20">
+    <row r="3" spans="1:23">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2897,7 +2277,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:20">
+    <row r="4" spans="1:23">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2956,7 +2336,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:20">
+    <row r="5" spans="1:23">
       <c r="A5">
         <v>3</v>
       </c>
@@ -3015,7 +2395,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:21">
+    <row r="6" spans="1:23">
       <c r="A6">
         <v>4</v>
       </c>
@@ -3050,10 +2430,10 @@
         <v>10</v>
       </c>
       <c r="M6">
-        <v>15000</v>
+        <v>150</v>
       </c>
       <c r="N6">
-        <v>6000</v>
+        <v>300</v>
       </c>
       <c r="O6">
         <v>50</v>
@@ -3077,7 +2457,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="7" spans="1:21">
+    <row r="7" spans="1:23">
       <c r="A7">
         <v>5</v>
       </c>
@@ -3139,7 +2519,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="1:20">
+    <row r="8" spans="1:23">
       <c r="A8">
         <v>6</v>
       </c>
@@ -3197,8 +2577,11 @@
       <c r="T8">
         <v>100</v>
       </c>
-    </row>
-    <row r="9" spans="1:21">
+      <c r="U8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23">
       <c r="A9">
         <v>7</v>
       </c>
@@ -3256,11 +2639,8 @@
       <c r="T9">
         <v>100</v>
       </c>
-      <c r="U9" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="10" spans="1:20">
+    </row>
+    <row r="10" spans="1:23">
       <c r="A10">
         <v>8</v>
       </c>
@@ -3319,7 +2699,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:20">
+    <row r="11" spans="1:23">
       <c r="A11">
         <v>9</v>
       </c>
@@ -3378,7 +2758,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="12" spans="1:20">
+    <row r="12" spans="1:23">
       <c r="A12">
         <v>10</v>
       </c>
@@ -3437,7 +2817,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:20">
+    <row r="13" spans="1:23">
       <c r="A13">
         <v>11</v>
       </c>
@@ -3496,7 +2876,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:20">
+    <row r="14" spans="1:23">
       <c r="A14">
         <v>12</v>
       </c>
@@ -3555,7 +2935,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:20">
+    <row r="15" spans="1:23">
       <c r="A15">
         <v>13</v>
       </c>
@@ -3614,7 +2994,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" spans="1:20">
+    <row r="16" spans="1:23">
       <c r="A16">
         <v>14</v>
       </c>
@@ -4086,44 +3466,42 @@
         <v>100</v>
       </c>
     </row>
-    <row r="24" spans="18:18">
+    <row r="24" spans="1:20">
       <c r="R24" s="1"/>
     </row>
-    <row r="25" spans="18:18">
+    <row r="25" spans="1:20">
       <c r="R25" s="1"/>
     </row>
-    <row r="26" spans="18:18">
+    <row r="26" spans="1:20">
       <c r="R26" s="1"/>
     </row>
-    <row r="27" spans="18:18">
+    <row r="27" spans="1:20">
       <c r="R27" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K32"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="10.425" style="1" customWidth="1"/>
-    <col min="2" max="2" width="23.2833333333333" style="1" customWidth="1"/>
-    <col min="3" max="3" width="27.7083333333333" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.1416666666667" style="1" customWidth="1"/>
-    <col min="5" max="5" width="8.14166666666667" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.425" style="1" customWidth="1"/>
-    <col min="7" max="7" width="6.85833333333333" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.2833333333333" style="1" customWidth="1"/>
-    <col min="9" max="9" width="15.5666666666667" style="1" customWidth="1"/>
-    <col min="10" max="11" width="16.8583333333333" style="1" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="6.85546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" style="1" customWidth="1"/>
+    <col min="10" max="11" width="16.85546875" style="1" customWidth="1"/>
     <col min="12" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:11">
+    <row r="1" spans="1:11" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4158,7 +3536,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="2" customHeight="1" spans="1:11">
+    <row r="2" spans="1:11" ht="30" customHeight="1">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -4190,7 +3568,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="3" customHeight="1" spans="1:11">
+    <row r="3" spans="1:11" ht="30" customHeight="1">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -4222,7 +3600,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="4" customHeight="1" spans="1:11">
+    <row r="4" spans="1:11" ht="30" customHeight="1">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -4254,7 +3632,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="5" customHeight="1" spans="1:11">
+    <row r="5" spans="1:11" ht="30" customHeight="1">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -4286,7 +3664,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="6" ht="33" customHeight="1" spans="1:11">
+    <row r="6" spans="1:11" ht="33" customHeight="1">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -4318,7 +3696,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="7" customHeight="1" spans="1:11">
+    <row r="7" spans="1:11" ht="30" customHeight="1">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -4350,7 +3728,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="8" customHeight="1" spans="1:11">
+    <row r="8" spans="1:11" ht="30" customHeight="1">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -4382,7 +3760,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="9" customHeight="1" spans="1:11">
+    <row r="9" spans="1:11" ht="30" customHeight="1">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -4414,7 +3792,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="10" customHeight="1" spans="1:11">
+    <row r="10" spans="1:11" ht="30" customHeight="1">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -4446,7 +3824,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="11" customHeight="1" spans="1:11">
+    <row r="11" spans="1:11" ht="30" customHeight="1">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -4478,7 +3856,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="12" customHeight="1" spans="1:11">
+    <row r="12" spans="1:11" ht="30" customHeight="1">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -4510,7 +3888,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="13" customHeight="1" spans="1:11">
+    <row r="13" spans="1:11" ht="30" customHeight="1">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -4533,7 +3911,7 @@
         <v>5</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="I13" s="9" t="s">
         <v>205</v>
@@ -4542,7 +3920,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="14" customHeight="1" spans="1:11">
+    <row r="14" spans="1:11" ht="30" customHeight="1">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -4565,7 +3943,7 @@
         <v>5</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="I14" s="9" t="s">
         <v>205</v>
@@ -4574,7 +3952,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="15" customHeight="1" spans="1:9">
+    <row r="15" spans="1:11" ht="30" customHeight="1">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -4603,7 +3981,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="16" ht="42" customHeight="1" spans="1:11">
+    <row r="16" spans="1:11" ht="42" customHeight="1">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -4635,7 +4013,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="17" customHeight="1" spans="1:11">
+    <row r="17" spans="1:11" ht="30" customHeight="1">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -4667,7 +4045,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="18" customHeight="1" spans="1:11">
+    <row r="18" spans="1:11" ht="30" customHeight="1">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -4699,7 +4077,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="19" customHeight="1" spans="1:9">
+    <row r="19" spans="1:11" ht="30" customHeight="1">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -4728,7 +4106,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="20" customHeight="1" spans="1:9">
+    <row r="20" spans="1:11" ht="30" customHeight="1">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -4757,7 +4135,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="21" customHeight="1" spans="1:9">
+    <row r="21" spans="1:11" ht="30" customHeight="1">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -4786,7 +4164,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="22" customHeight="1" spans="1:11">
+    <row r="22" spans="1:11" ht="30" customHeight="1">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -4818,7 +4196,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="23" customHeight="1" spans="1:11">
+    <row r="23" spans="1:11" ht="30" customHeight="1">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -4850,7 +4228,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="24" customHeight="1" spans="1:11">
+    <row r="24" spans="1:11" ht="30" customHeight="1">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -4882,7 +4260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" customHeight="1" spans="1:11">
+    <row r="25" spans="1:11" ht="30" customHeight="1">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -4914,7 +4292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" customHeight="1" spans="1:11">
+    <row r="26" spans="1:11" ht="30" customHeight="1">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -4928,7 +4306,7 @@
         <v>237</v>
       </c>
       <c r="E26" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>101</v>
@@ -4946,7 +4324,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="27" customHeight="1" spans="1:11">
+    <row r="27" spans="1:11" ht="30" customHeight="1">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -4960,7 +4338,7 @@
         <v>237</v>
       </c>
       <c r="E27" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>101</v>
@@ -4978,7 +4356,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="28" customHeight="1" spans="1:11">
+    <row r="28" spans="1:11" ht="30" customHeight="1">
       <c r="A28" s="1">
         <v>26</v>
       </c>
@@ -4992,7 +4370,7 @@
         <v>237</v>
       </c>
       <c r="E28" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>101</v>
@@ -5010,7 +4388,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="29" customHeight="1" spans="1:11">
+    <row r="29" spans="1:11" ht="30" customHeight="1">
       <c r="A29" s="1">
         <v>27</v>
       </c>
@@ -5024,7 +4402,7 @@
         <v>237</v>
       </c>
       <c r="E29" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>101</v>
@@ -5042,7 +4420,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="30" customHeight="1" spans="1:11">
+    <row r="30" spans="1:11" ht="30" customHeight="1">
       <c r="A30" s="1">
         <v>28</v>
       </c>
@@ -5056,7 +4434,7 @@
         <v>237</v>
       </c>
       <c r="E30" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>101</v>
@@ -5074,7 +4452,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="31" customHeight="1" spans="1:9">
+    <row r="31" spans="1:11" ht="30" customHeight="1">
       <c r="A31" s="1">
         <v>29</v>
       </c>
@@ -5088,7 +4466,7 @@
         <v>237</v>
       </c>
       <c r="E31" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>101</v>
@@ -5103,7 +4481,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="32" customHeight="1" spans="1:9">
+    <row r="32" spans="1:11" ht="30" customHeight="1">
       <c r="A32" s="1">
         <v>30</v>
       </c>
@@ -5131,21 +4509,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="17.2833333333333" customWidth="1"/>
-    <col min="4" max="4" width="20.1416666666667" customWidth="1"/>
-    <col min="5" max="5" width="19.7083333333333" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" customWidth="1"/>
+    <col min="5" max="5" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -5293,21 +4669,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultColWidth="8.70833333333333" defaultRowHeight="14" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.14166666666667" customWidth="1"/>
-    <col min="2" max="2" width="6.70833333333333" customWidth="1"/>
-    <col min="3" max="3" width="10.425" customWidth="1"/>
-    <col min="4" max="4" width="5.70833333333333" customWidth="1"/>
-    <col min="5" max="5" width="11.425" customWidth="1"/>
+    <col min="1" max="1" width="3.140625" customWidth="1"/>
+    <col min="2" max="2" width="6.7109375" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" customWidth="1"/>
+    <col min="4" max="4" width="5.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -5329,6 +4703,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added icon in excels
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Raising.xlsx
+++ b/Assets/StreamingAssets/Configurations/Raising.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8219726-2132-4B29-9A26-9311D49AF6C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="22190" windowHeight="9040" activeTab="2"/>
+    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingEffects" sheetId="1" r:id="rId1"/>
@@ -25,8 +31,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -1226,18 +1230,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="21">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -1247,152 +1245,8 @@
       <name val="宋体"/>
       <charset val="134"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="41">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1425,7 +1279,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.0999786370433668"/>
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1447,194 +1301,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1642,251 +1310,9 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1930,70 +1356,26 @@
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="000BF30B"/>
-      <color rgb="00E3A7F7"/>
-      <color rgb="00F567ED"/>
-      <color rgb="00DEBA2C"/>
-      <color rgb="00FD460D"/>
+      <color rgb="FF0BF30B"/>
+      <color rgb="FFE3A7F7"/>
+      <color rgb="FFF567ED"/>
+      <color rgb="FFDEBA2C"/>
+      <color rgb="FFFD460D"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -2251,22 +1633,22 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F56"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.425" customWidth="1"/>
-    <col min="2" max="2" width="31.425" customWidth="1"/>
-    <col min="3" max="3" width="29.425" customWidth="1"/>
-    <col min="4" max="4" width="31.7083333333333" customWidth="1"/>
-    <col min="5" max="5" width="15.2833333333333" customWidth="1"/>
-    <col min="6" max="6" width="29.5666666666667" customWidth="1"/>
-    <col min="7" max="7" width="15.7083333333333" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="31.42578125" customWidth="1"/>
+    <col min="3" max="3" width="29.42578125" customWidth="1"/>
+    <col min="4" max="4" width="31.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" customWidth="1"/>
+    <col min="6" max="6" width="29.5703125" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -2400,7 +1782,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:6">
       <c r="A8">
         <v>6</v>
       </c>
@@ -2414,7 +1796,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:6">
       <c r="A9">
         <v>7</v>
       </c>
@@ -2428,7 +1810,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:6">
       <c r="A10">
         <v>8</v>
       </c>
@@ -2612,7 +1994,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:6">
       <c r="A21">
         <v>19</v>
       </c>
@@ -2626,7 +2008,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:6">
       <c r="A22">
         <v>20</v>
       </c>
@@ -2637,7 +2019,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:6">
       <c r="A23">
         <v>21</v>
       </c>
@@ -2665,7 +2047,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:6">
       <c r="A25">
         <v>23</v>
       </c>
@@ -2699,7 +2081,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:6">
       <c r="A27">
         <v>25</v>
       </c>
@@ -2894,7 +2276,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:6">
       <c r="A39">
         <v>37</v>
       </c>
@@ -2967,7 +2349,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="44" spans="1:4">
+    <row r="44" spans="1:6">
       <c r="A44">
         <v>42</v>
       </c>
@@ -3051,7 +2433,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="50" spans="1:4">
+    <row r="50" spans="1:6">
       <c r="A50">
         <v>48</v>
       </c>
@@ -3062,7 +2444,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="51" spans="1:4">
+    <row r="51" spans="1:6">
       <c r="A51">
         <v>49</v>
       </c>
@@ -3073,7 +2455,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="52" spans="1:4">
+    <row r="52" spans="1:6">
       <c r="A52">
         <v>50</v>
       </c>
@@ -3084,7 +2466,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="53" spans="1:4">
+    <row r="53" spans="1:6">
       <c r="A53">
         <v>51</v>
       </c>
@@ -3095,7 +2477,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="54" spans="1:4">
+    <row r="54" spans="1:6">
       <c r="A54">
         <v>52</v>
       </c>
@@ -3106,7 +2488,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="55" spans="1:4">
+    <row r="55" spans="1:6">
       <c r="A55">
         <v>53</v>
       </c>
@@ -3117,7 +2499,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="56" spans="1:4">
+    <row r="56" spans="1:6">
       <c r="A56">
         <v>54</v>
       </c>
@@ -3130,35 +2512,33 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:W27"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.425" customWidth="1"/>
-    <col min="2" max="2" width="21.8583333333333" customWidth="1"/>
-    <col min="3" max="3" width="22.2833333333333" customWidth="1"/>
-    <col min="4" max="4" width="11.5666666666667" customWidth="1"/>
-    <col min="5" max="6" width="11.425" customWidth="1"/>
-    <col min="7" max="7" width="6.70833333333333" customWidth="1"/>
-    <col min="9" max="9" width="8.14166666666667" customWidth="1"/>
-    <col min="10" max="10" width="15.425" customWidth="1"/>
-    <col min="11" max="11" width="10.7083333333333" customWidth="1"/>
-    <col min="12" max="12" width="3.28333333333333" customWidth="1"/>
-    <col min="13" max="13" width="6.425" customWidth="1"/>
-    <col min="14" max="14" width="11.7083333333333" customWidth="1"/>
-    <col min="15" max="15" width="10.2833333333333" customWidth="1"/>
-    <col min="16" max="16" width="10.7083333333333" customWidth="1"/>
-    <col min="17" max="17" width="11.8583333333333" customWidth="1"/>
-    <col min="18" max="18" width="8.28333333333333" customWidth="1"/>
-    <col min="19" max="19" width="10.1416666666667" customWidth="1"/>
-    <col min="20" max="20" width="14.1416666666667" customWidth="1"/>
-    <col min="21" max="21" width="10.2833333333333" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" customWidth="1"/>
+    <col min="3" max="3" width="22.28515625" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" customWidth="1"/>
+    <col min="5" max="6" width="11.42578125" customWidth="1"/>
+    <col min="7" max="7" width="6.7109375" customWidth="1"/>
+    <col min="9" max="9" width="8.140625" customWidth="1"/>
+    <col min="10" max="10" width="15.42578125" customWidth="1"/>
+    <col min="11" max="11" width="10.7109375" customWidth="1"/>
+    <col min="12" max="12" width="3.28515625" customWidth="1"/>
+    <col min="13" max="13" width="6.42578125" customWidth="1"/>
+    <col min="14" max="14" width="11.7109375" customWidth="1"/>
+    <col min="15" max="15" width="10.28515625" customWidth="1"/>
+    <col min="16" max="16" width="10.7109375" customWidth="1"/>
+    <col min="17" max="17" width="11.85546875" customWidth="1"/>
+    <col min="18" max="18" width="8.28515625" customWidth="1"/>
+    <col min="19" max="19" width="10.140625" customWidth="1"/>
+    <col min="20" max="20" width="14.140625" customWidth="1"/>
+    <col min="21" max="21" width="10.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -3232,7 +2612,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="2" spans="1:20">
+    <row r="2" spans="1:23">
       <c r="A2">
         <v>0</v>
       </c>
@@ -3291,7 +2671,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:20">
+    <row r="3" spans="1:23">
       <c r="A3">
         <v>1</v>
       </c>
@@ -3350,7 +2730,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:20">
+    <row r="4" spans="1:23">
       <c r="A4">
         <v>2</v>
       </c>
@@ -3409,7 +2789,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:20">
+    <row r="5" spans="1:23">
       <c r="A5">
         <v>3</v>
       </c>
@@ -3468,7 +2848,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:21">
+    <row r="6" spans="1:23">
       <c r="A6">
         <v>4</v>
       </c>
@@ -3530,7 +2910,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="7" spans="1:21">
+    <row r="7" spans="1:23">
       <c r="A7">
         <v>5</v>
       </c>
@@ -3592,7 +2972,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="8" spans="1:21">
+    <row r="8" spans="1:23">
       <c r="A8">
         <v>6</v>
       </c>
@@ -3654,7 +3034,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="9" spans="1:21">
+    <row r="9" spans="1:23">
       <c r="A9">
         <v>7</v>
       </c>
@@ -3716,7 +3096,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="10" spans="1:21">
+    <row r="10" spans="1:23">
       <c r="A10">
         <v>8</v>
       </c>
@@ -3778,7 +3158,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="11" spans="1:21">
+    <row r="11" spans="1:23">
       <c r="A11">
         <v>9</v>
       </c>
@@ -3840,7 +3220,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="12" spans="1:21">
+    <row r="12" spans="1:23">
       <c r="A12">
         <v>10</v>
       </c>
@@ -3902,7 +3282,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="13" spans="1:21">
+    <row r="13" spans="1:23">
       <c r="A13">
         <v>11</v>
       </c>
@@ -3964,7 +3344,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="14" spans="1:21">
+    <row r="14" spans="1:23">
       <c r="A14">
         <v>12</v>
       </c>
@@ -4026,7 +3406,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="15" spans="1:21">
+    <row r="15" spans="1:23">
       <c r="A15">
         <v>13</v>
       </c>
@@ -4088,7 +3468,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="16" spans="1:22">
+    <row r="16" spans="1:23">
       <c r="A16">
         <v>14</v>
       </c>
@@ -4153,7 +3533,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="17" spans="1:21">
+    <row r="17" spans="1:22">
       <c r="A17">
         <v>15</v>
       </c>
@@ -4215,7 +3595,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="18" spans="1:21">
+    <row r="18" spans="1:22">
       <c r="A18">
         <v>16</v>
       </c>
@@ -4277,7 +3657,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="19" spans="1:21">
+    <row r="19" spans="1:22">
       <c r="A19">
         <v>17</v>
       </c>
@@ -4469,7 +3849,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="22" spans="1:20">
+    <row r="22" spans="1:22">
       <c r="A22">
         <v>20</v>
       </c>
@@ -4528,7 +3908,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="23" spans="1:21">
+    <row r="23" spans="1:22">
       <c r="A23">
         <v>21</v>
       </c>
@@ -4590,44 +3970,42 @@
         <v>199</v>
       </c>
     </row>
-    <row r="24" spans="18:18">
+    <row r="24" spans="1:22">
       <c r="R24" s="1"/>
     </row>
-    <row r="25" spans="18:18">
+    <row r="25" spans="1:22">
       <c r="R25" s="1"/>
     </row>
-    <row r="26" spans="18:18">
+    <row r="26" spans="1:22">
       <c r="R26" s="1"/>
     </row>
-    <row r="27" spans="18:18">
+    <row r="27" spans="1:22">
       <c r="R27" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K54"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="10.425" style="1" customWidth="1"/>
-    <col min="2" max="2" width="23.2833333333333" style="1" customWidth="1"/>
-    <col min="3" max="3" width="27.7083333333333" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.1416666666667" style="1" customWidth="1"/>
-    <col min="5" max="5" width="8.14166666666667" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.425" style="1" customWidth="1"/>
-    <col min="7" max="7" width="6.85833333333333" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.2833333333333" style="1" customWidth="1"/>
-    <col min="9" max="9" width="15.5666666666667" style="1" customWidth="1"/>
-    <col min="10" max="11" width="16.8583333333333" style="1" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="6.85546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" style="1" customWidth="1"/>
+    <col min="10" max="11" width="16.85546875" style="1" customWidth="1"/>
     <col min="12" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:11">
+    <row r="1" spans="1:11" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4662,7 +4040,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" customHeight="1" spans="1:11">
+    <row r="2" spans="1:11" ht="30" customHeight="1">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -4694,7 +4072,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="3" customHeight="1" spans="1:11">
+    <row r="3" spans="1:11" ht="30" customHeight="1">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -4726,7 +4104,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="4" customHeight="1" spans="1:11">
+    <row r="4" spans="1:11" ht="30" customHeight="1">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -4758,7 +4136,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="5" customHeight="1" spans="1:11">
+    <row r="5" spans="1:11" ht="30" customHeight="1">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -4790,7 +4168,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="6" ht="33" customHeight="1" spans="1:11">
+    <row r="6" spans="1:11" ht="33" customHeight="1">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -4822,7 +4200,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="7" customHeight="1" spans="1:11">
+    <row r="7" spans="1:11" ht="30" customHeight="1">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -4854,7 +4232,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="8" customHeight="1" spans="1:11">
+    <row r="8" spans="1:11" ht="30" customHeight="1">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -4886,7 +4264,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="9" customHeight="1" spans="1:11">
+    <row r="9" spans="1:11" ht="30" customHeight="1">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -4918,7 +4296,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="10" customHeight="1" spans="1:11">
+    <row r="10" spans="1:11" ht="30" customHeight="1">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -4950,7 +4328,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="11" customHeight="1" spans="1:11">
+    <row r="11" spans="1:11" ht="30" customHeight="1">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -4982,7 +4360,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="12" customHeight="1" spans="1:11">
+    <row r="12" spans="1:11" ht="30" customHeight="1">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -5014,7 +4392,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="13" customHeight="1" spans="1:11">
+    <row r="13" spans="1:11" ht="30" customHeight="1">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -5042,12 +4420,11 @@
       <c r="I13" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="J13" s="1"/>
       <c r="K13" s="1" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="14" customHeight="1" spans="1:11">
+    <row r="14" spans="1:11" ht="30" customHeight="1">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -5079,7 +4456,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="15" customHeight="1" spans="1:11">
+    <row r="15" spans="1:11" ht="30" customHeight="1">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -5107,12 +4484,11 @@
       <c r="I15" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="J15" s="1"/>
       <c r="K15" s="1" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="16" ht="42" customHeight="1" spans="1:11">
+    <row r="16" spans="1:11" ht="42" customHeight="1">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -5142,7 +4518,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="17" customHeight="1" spans="1:11">
+    <row r="17" spans="1:11" ht="30" customHeight="1">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -5172,7 +4548,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="18" customHeight="1" spans="1:11">
+    <row r="18" spans="1:11" ht="30" customHeight="1">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -5202,7 +4578,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="19" customHeight="1" spans="1:11">
+    <row r="19" spans="1:11" ht="30" customHeight="1">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -5234,7 +4610,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="20" customHeight="1" spans="1:11">
+    <row r="20" spans="1:11" ht="30" customHeight="1">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -5266,7 +4642,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="21" customHeight="1" spans="1:11">
+    <row r="21" spans="1:11" ht="30" customHeight="1">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -5298,7 +4674,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="22" customHeight="1" spans="1:11">
+    <row r="22" spans="1:11" ht="30" customHeight="1">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -5330,7 +4706,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="23" customHeight="1" spans="1:11">
+    <row r="23" spans="1:11" ht="30" customHeight="1">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -5362,7 +4738,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="24" customHeight="1" spans="1:11">
+    <row r="24" spans="1:11" ht="30" customHeight="1">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -5394,7 +4770,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="25" customHeight="1" spans="1:11">
+    <row r="25" spans="1:11" ht="30" customHeight="1">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -5426,7 +4802,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="26" customHeight="1" spans="1:11">
+    <row r="26" spans="1:11" ht="30" customHeight="1">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -5458,7 +4834,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="27" customHeight="1" spans="1:11">
+    <row r="27" spans="1:11" ht="30" customHeight="1">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -5490,7 +4866,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="28" customHeight="1" spans="1:11">
+    <row r="28" spans="1:11" ht="30" customHeight="1">
       <c r="A28" s="1">
         <v>26</v>
       </c>
@@ -5522,7 +4898,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="29" customHeight="1" spans="1:11">
+    <row r="29" spans="1:11" ht="30" customHeight="1">
       <c r="A29" s="1">
         <v>27</v>
       </c>
@@ -5554,7 +4930,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="30" customHeight="1" spans="1:11">
+    <row r="30" spans="1:11" ht="30" customHeight="1">
       <c r="A30" s="1">
         <v>28</v>
       </c>
@@ -5586,7 +4962,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="31" customHeight="1" spans="1:9">
+    <row r="31" spans="1:11" ht="30" customHeight="1">
       <c r="A31" s="1">
         <v>29</v>
       </c>
@@ -5615,7 +4991,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="32" customHeight="1" spans="1:11">
+    <row r="32" spans="1:11" ht="30" customHeight="1">
       <c r="A32" s="1">
         <v>30</v>
       </c>
@@ -5644,7 +5020,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="33" customHeight="1" spans="1:11">
+    <row r="33" spans="1:11" ht="30" customHeight="1">
       <c r="A33" s="1">
         <v>31</v>
       </c>
@@ -5676,7 +5052,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="34" customHeight="1" spans="1:11">
+    <row r="34" spans="1:11" ht="30" customHeight="1">
       <c r="A34" s="1">
         <v>32</v>
       </c>
@@ -5708,7 +5084,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="35" customHeight="1" spans="1:11">
+    <row r="35" spans="1:11" ht="30" customHeight="1">
       <c r="A35" s="1">
         <v>33</v>
       </c>
@@ -5740,7 +5116,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="36" customHeight="1" spans="1:11">
+    <row r="36" spans="1:11" ht="30" customHeight="1">
       <c r="A36" s="1">
         <v>34</v>
       </c>
@@ -5772,7 +5148,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="37" customHeight="1" spans="1:11">
+    <row r="37" spans="1:11" ht="30" customHeight="1">
       <c r="A37" s="1">
         <v>35</v>
       </c>
@@ -5804,7 +5180,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="38" customHeight="1" spans="1:11">
+    <row r="38" spans="1:11" ht="30" customHeight="1">
       <c r="A38" s="1">
         <v>36</v>
       </c>
@@ -5836,7 +5212,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="39" customHeight="1" spans="1:11">
+    <row r="39" spans="1:11" ht="30" customHeight="1">
       <c r="A39" s="1">
         <v>37</v>
       </c>
@@ -5868,7 +5244,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="40" customHeight="1" spans="1:11">
+    <row r="40" spans="1:11" ht="30" customHeight="1">
       <c r="A40" s="1">
         <v>38</v>
       </c>
@@ -5900,7 +5276,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="41" customHeight="1" spans="1:11">
+    <row r="41" spans="1:11" ht="30" customHeight="1">
       <c r="A41" s="1">
         <v>39</v>
       </c>
@@ -5932,7 +5308,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="42" customHeight="1" spans="1:11">
+    <row r="42" spans="1:11" ht="30" customHeight="1">
       <c r="A42" s="1">
         <v>40</v>
       </c>
@@ -5964,7 +5340,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="43" customHeight="1" spans="1:11">
+    <row r="43" spans="1:11" ht="30" customHeight="1">
       <c r="A43" s="1">
         <v>41</v>
       </c>
@@ -5996,7 +5372,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="44" customHeight="1" spans="1:11">
+    <row r="44" spans="1:11" ht="30" customHeight="1">
       <c r="A44" s="1">
         <v>42</v>
       </c>
@@ -6028,7 +5404,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="45" customHeight="1" spans="1:11">
+    <row r="45" spans="1:11" ht="30" customHeight="1">
       <c r="A45" s="1">
         <v>43</v>
       </c>
@@ -6060,7 +5436,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="46" customHeight="1" spans="1:9">
+    <row r="46" spans="1:11" ht="30" customHeight="1">
       <c r="A46" s="1">
         <v>44</v>
       </c>
@@ -6089,7 +5465,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="47" customHeight="1" spans="1:9">
+    <row r="47" spans="1:11" ht="30" customHeight="1">
       <c r="A47" s="1">
         <v>45</v>
       </c>
@@ -6118,7 +5494,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="48" customHeight="1" spans="1:9">
+    <row r="48" spans="1:11" ht="30" customHeight="1">
       <c r="A48" s="1">
         <v>46</v>
       </c>
@@ -6147,7 +5523,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="49" customHeight="1" spans="1:9">
+    <row r="49" spans="1:11" ht="30" customHeight="1">
       <c r="A49" s="1">
         <v>47</v>
       </c>
@@ -6176,7 +5552,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="50" customHeight="1" spans="1:10">
+    <row r="50" spans="1:11" ht="30" customHeight="1">
       <c r="A50" s="1">
         <v>48</v>
       </c>
@@ -6208,7 +5584,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="51" customHeight="1" spans="1:10">
+    <row r="51" spans="1:11" ht="30" customHeight="1">
       <c r="A51" s="1">
         <v>49</v>
       </c>
@@ -6240,7 +5616,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52" customHeight="1" spans="1:10">
+    <row r="52" spans="1:11" ht="30" customHeight="1">
       <c r="A52" s="1">
         <v>50</v>
       </c>
@@ -6272,7 +5648,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="53" customHeight="1" spans="1:10">
+    <row r="53" spans="1:11" ht="30" customHeight="1">
       <c r="A53" s="1">
         <v>51</v>
       </c>
@@ -6304,7 +5680,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="54" customHeight="1" spans="1:11">
+    <row r="54" spans="1:11" ht="30" customHeight="1">
       <c r="A54" s="1">
         <v>52</v>
       </c>
@@ -6338,21 +5714,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="17.2833333333333" customWidth="1"/>
-    <col min="4" max="4" width="20.1416666666667" customWidth="1"/>
-    <col min="5" max="5" width="19.7083333333333" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" customWidth="1"/>
+    <col min="5" max="5" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -6514,21 +5888,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultColWidth="8.70833333333333" defaultRowHeight="14" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.14166666666667" customWidth="1"/>
-    <col min="2" max="2" width="6.70833333333333" customWidth="1"/>
-    <col min="3" max="3" width="10.425" customWidth="1"/>
-    <col min="4" max="4" width="5.70833333333333" customWidth="1"/>
-    <col min="5" max="5" width="11.425" customWidth="1"/>
+    <col min="1" max="1" width="3.140625" customWidth="1"/>
+    <col min="2" max="2" width="6.7109375" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" customWidth="1"/>
+    <col min="4" max="4" width="5.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -6690,6 +6062,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fixed score exceeding rating level max value
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Raising.xlsx
+++ b/Assets/StreamingAssets/Configurations/Raising.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8356CAAA-2926-4422-871D-17CA6F9E6620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F963974E-9A89-49EF-AE3C-086BDE255F12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingEffects" sheetId="1" r:id="rId1"/>
@@ -31,8 +31,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>

</xml_diff>

<commit_message>
fixing scheduling conditions reading
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Raising.xlsx
+++ b/Assets/StreamingAssets/Configurations/Raising.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BD3CC5B-9659-49D7-9518-C821738468F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{957B0E88-4ACD-42F4-8081-C659BA3BA5B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingEffects" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1008" uniqueCount="480">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1005" uniqueCount="479">
   <si>
     <t>ID</t>
   </si>
@@ -1491,9 +1491,6 @@
   </si>
   <si>
     <t>UDLR</t>
-  </si>
-  <si>
-    <t>All</t>
   </si>
 </sst>
 </file>
@@ -7188,15 +7185,6 @@
       <c r="D3">
         <v>2</v>
       </c>
-      <c r="E3" t="s">
-        <v>479</v>
-      </c>
-      <c r="F3" t="s">
-        <v>3</v>
-      </c>
-      <c r="G3" t="s">
-        <v>235</v>
-      </c>
       <c r="H3">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
character, schedule save data
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Raising.xlsx
+++ b/Assets/StreamingAssets/Configurations/Raising.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{243AA553-5900-4C5F-89B9-9045C581CCC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{774C0E2D-41E9-497A-9F8C-CFD7B772E3CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingEffects" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
added events without dialogs
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Raising.xlsx
+++ b/Assets/StreamingAssets/Configurations/Raising.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{774C0E2D-41E9-497A-9F8C-CFD7B772E3CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{771A089A-8506-4DB1-A95C-2B762FC7ACBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingEffects" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1005" uniqueCount="479">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="483">
   <si>
     <t>ID</t>
   </si>
@@ -1491,6 +1491,18 @@
   </si>
   <si>
     <t>UDLR</t>
+  </si>
+  <si>
+    <t>Effect4</t>
+  </si>
+  <si>
+    <t>E4Param</t>
+  </si>
+  <si>
+    <t>Effect5</t>
+  </si>
+  <si>
+    <t>E5Param</t>
   </si>
 </sst>
 </file>
@@ -4411,7 +4423,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:L75"/>
+  <dimension ref="A1:V75"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="30" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="1" customWidth="1"/>
@@ -4429,7 +4441,7 @@
     <col min="13" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="30" customHeight="1">
+    <row r="1" spans="1:22" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4466,8 +4478,38 @@
       <c r="L1" s="1" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" ht="30" customHeight="1">
+      <c r="M1" s="14" t="s">
+        <v>471</v>
+      </c>
+      <c r="N1" t="s">
+        <v>472</v>
+      </c>
+      <c r="O1" s="14" t="s">
+        <v>473</v>
+      </c>
+      <c r="P1" t="s">
+        <v>474</v>
+      </c>
+      <c r="Q1" s="14" t="s">
+        <v>475</v>
+      </c>
+      <c r="R1" t="s">
+        <v>476</v>
+      </c>
+      <c r="S1" s="14" t="s">
+        <v>479</v>
+      </c>
+      <c r="T1" t="s">
+        <v>480</v>
+      </c>
+      <c r="U1" s="14" t="s">
+        <v>481</v>
+      </c>
+      <c r="V1" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" ht="30" customHeight="1">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -4502,7 +4544,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="30" customHeight="1">
+    <row r="3" spans="1:22" ht="30" customHeight="1">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -4537,7 +4579,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="30" customHeight="1">
+    <row r="4" spans="1:22" ht="30" customHeight="1">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -4569,7 +4611,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="30" customHeight="1">
+    <row r="5" spans="1:22" ht="30" customHeight="1">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -4601,7 +4643,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="33" customHeight="1">
+    <row r="6" spans="1:22" ht="33" customHeight="1">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -4633,7 +4675,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="30" customHeight="1">
+    <row r="7" spans="1:22" ht="30" customHeight="1">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -4665,7 +4707,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="30" customHeight="1">
+    <row r="8" spans="1:22" ht="30" customHeight="1">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -4697,7 +4739,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="30" customHeight="1">
+    <row r="9" spans="1:22" ht="30" customHeight="1">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -4729,7 +4771,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="30" customHeight="1">
+    <row r="10" spans="1:22" ht="30" customHeight="1">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -4761,7 +4803,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="30" customHeight="1">
+    <row r="11" spans="1:22" ht="30" customHeight="1">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -4793,7 +4835,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="30" customHeight="1">
+    <row r="12" spans="1:22" ht="30" customHeight="1">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -4825,7 +4867,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="30" customHeight="1">
+    <row r="13" spans="1:22" ht="30" customHeight="1">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -4857,7 +4899,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="30" customHeight="1">
+    <row r="14" spans="1:22" ht="30" customHeight="1">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -4889,7 +4931,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="30" customHeight="1">
+    <row r="15" spans="1:22" ht="30" customHeight="1">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -4921,7 +4963,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="42" customHeight="1">
+    <row r="16" spans="1:22" ht="42" customHeight="1">
       <c r="A16" s="1">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Raising Animation System 1
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Raising.xlsx
+++ b/Assets/StreamingAssets/Configurations/Raising.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9DB62DB-5781-4004-915C-10D028310E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="30720" windowHeight="13380" activeTab="1"/>
+    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingEffects" sheetId="1" r:id="rId1"/>
@@ -26,8 +32,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -35,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1051" uniqueCount="504">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1052" uniqueCount="505">
   <si>
     <t>ID</t>
   </si>
@@ -1572,23 +1576,20 @@
   </si>
   <si>
     <t>LR</t>
+  </si>
+  <si>
+    <t>在事件前执行</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="21">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -1598,152 +1599,8 @@
       <name val="宋体"/>
       <charset val="134"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="42">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1776,7 +1633,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.0999786370433668"/>
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1804,194 +1661,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -2008,251 +1679,9 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -2303,72 +1732,28 @@
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="000BF30B"/>
-      <color rgb="00E3A7F7"/>
-      <color rgb="00F567ED"/>
-      <color rgb="00DEBA2C"/>
-      <color rgb="00FD460D"/>
-      <color rgb="00A122FB"/>
-      <color rgb="004C8BFE"/>
+      <color rgb="FF0BF30B"/>
+      <color rgb="FFE3A7F7"/>
+      <color rgb="FFF567ED"/>
+      <color rgb="FFDEBA2C"/>
+      <color rgb="FFFD460D"/>
+      <color rgb="FFA122FB"/>
+      <color rgb="FF4C8BFE"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -2626,22 +2011,22 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F66"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.42592592592593" customWidth="1"/>
-    <col min="2" max="2" width="31.4259259259259" customWidth="1"/>
-    <col min="3" max="3" width="29.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="31.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="15.287037037037" customWidth="1"/>
-    <col min="6" max="6" width="29.5740740740741" customWidth="1"/>
-    <col min="7" max="7" width="15.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="31.42578125" customWidth="1"/>
+    <col min="3" max="3" width="29.42578125" customWidth="1"/>
+    <col min="4" max="4" width="31.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" customWidth="1"/>
+    <col min="6" max="6" width="29.5703125" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -2775,7 +2160,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:6">
       <c r="A8">
         <v>6</v>
       </c>
@@ -2789,7 +2174,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:6">
       <c r="A9">
         <v>7</v>
       </c>
@@ -2803,7 +2188,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:6">
       <c r="A10">
         <v>8</v>
       </c>
@@ -2987,7 +2372,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:6">
       <c r="A21">
         <v>19</v>
       </c>
@@ -3001,7 +2386,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:6">
       <c r="A22">
         <v>20</v>
       </c>
@@ -3012,7 +2397,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:6">
       <c r="A23">
         <v>21</v>
       </c>
@@ -3040,7 +2425,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:6">
       <c r="A25">
         <v>23</v>
       </c>
@@ -3074,7 +2459,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:6">
       <c r="A27">
         <v>25</v>
       </c>
@@ -3269,7 +2654,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:6">
       <c r="A39">
         <v>37</v>
       </c>
@@ -3348,7 +2733,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="44" spans="1:4">
+    <row r="44" spans="1:6">
       <c r="A44">
         <v>42</v>
       </c>
@@ -3432,7 +2817,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="50" spans="1:4">
+    <row r="50" spans="1:6">
       <c r="A50">
         <v>48</v>
       </c>
@@ -3443,7 +2828,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="51" spans="1:4">
+    <row r="51" spans="1:6">
       <c r="A51">
         <v>49</v>
       </c>
@@ -3454,7 +2839,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="52" spans="1:4">
+    <row r="52" spans="1:6">
       <c r="A52">
         <v>50</v>
       </c>
@@ -3465,7 +2850,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="53" spans="1:4">
+    <row r="53" spans="1:6">
       <c r="A53">
         <v>51</v>
       </c>
@@ -3476,7 +2861,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="54" spans="1:4">
+    <row r="54" spans="1:6">
       <c r="A54">
         <v>52</v>
       </c>
@@ -3487,7 +2872,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="55" spans="1:4">
+    <row r="55" spans="1:6">
       <c r="A55">
         <v>53</v>
       </c>
@@ -3498,7 +2883,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="56" spans="1:4">
+    <row r="56" spans="1:6">
       <c r="A56">
         <v>54</v>
       </c>
@@ -3523,7 +2908,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="58" spans="1:4">
+    <row r="58" spans="1:6">
       <c r="A58">
         <v>56</v>
       </c>
@@ -3621,7 +3006,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="65" spans="1:4">
+    <row r="65" spans="1:6">
       <c r="A65">
         <v>63</v>
       </c>
@@ -3648,36 +3033,34 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:X27"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.42592592592593" customWidth="1"/>
-    <col min="2" max="2" width="21.8518518518519" customWidth="1"/>
-    <col min="3" max="3" width="22.287037037037" customWidth="1"/>
-    <col min="4" max="4" width="11.5740740740741" customWidth="1"/>
-    <col min="5" max="6" width="11.4259259259259" customWidth="1"/>
-    <col min="7" max="7" width="6.71296296296296" customWidth="1"/>
-    <col min="9" max="9" width="8.13888888888889" customWidth="1"/>
-    <col min="10" max="11" width="15.4259259259259" customWidth="1"/>
-    <col min="12" max="12" width="10.712962962963" customWidth="1"/>
-    <col min="13" max="13" width="3.28703703703704" customWidth="1"/>
-    <col min="14" max="14" width="6.42592592592593" customWidth="1"/>
-    <col min="15" max="15" width="11.712962962963" customWidth="1"/>
-    <col min="16" max="16" width="10.287037037037" customWidth="1"/>
-    <col min="17" max="17" width="10.712962962963" customWidth="1"/>
-    <col min="18" max="18" width="11.8518518518519" customWidth="1"/>
-    <col min="19" max="19" width="8.28703703703704" customWidth="1"/>
-    <col min="20" max="20" width="10.1388888888889" customWidth="1"/>
-    <col min="21" max="21" width="14.1388888888889" customWidth="1"/>
-    <col min="22" max="22" width="10.287037037037" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" customWidth="1"/>
+    <col min="3" max="3" width="22.28515625" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" customWidth="1"/>
+    <col min="5" max="6" width="11.42578125" customWidth="1"/>
+    <col min="7" max="7" width="6.7109375" customWidth="1"/>
+    <col min="9" max="9" width="8.140625" customWidth="1"/>
+    <col min="10" max="11" width="15.42578125" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" customWidth="1"/>
+    <col min="13" max="13" width="3.28515625" customWidth="1"/>
+    <col min="14" max="14" width="6.42578125" customWidth="1"/>
+    <col min="15" max="15" width="11.7109375" customWidth="1"/>
+    <col min="16" max="16" width="10.28515625" customWidth="1"/>
+    <col min="17" max="17" width="10.7109375" customWidth="1"/>
+    <col min="18" max="18" width="11.85546875" customWidth="1"/>
+    <col min="19" max="19" width="8.28515625" customWidth="1"/>
+    <col min="20" max="20" width="10.140625" customWidth="1"/>
+    <col min="21" max="21" width="14.140625" customWidth="1"/>
+    <col min="22" max="22" width="10.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24">
@@ -3754,7 +3137,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="2" ht="41.4" spans="1:21">
+    <row r="2" spans="1:24" ht="60">
       <c r="A2">
         <v>0</v>
       </c>
@@ -3816,7 +3199,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" ht="41.4" spans="1:21">
+    <row r="3" spans="1:24" ht="60">
       <c r="A3">
         <v>1</v>
       </c>
@@ -3878,7 +3261,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" ht="41.4" spans="1:21">
+    <row r="4" spans="1:24" ht="60">
       <c r="A4">
         <v>2</v>
       </c>
@@ -3940,7 +3323,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:21">
+    <row r="5" spans="1:24">
       <c r="A5">
         <v>3</v>
       </c>
@@ -3999,7 +3382,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:22">
+    <row r="6" spans="1:24">
       <c r="A6">
         <v>4</v>
       </c>
@@ -4061,7 +3444,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="7" spans="1:22">
+    <row r="7" spans="1:24">
       <c r="A7">
         <v>5</v>
       </c>
@@ -4123,7 +3506,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="8" spans="1:22">
+    <row r="8" spans="1:24">
       <c r="A8">
         <v>6</v>
       </c>
@@ -4185,7 +3568,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="9" spans="1:22">
+    <row r="9" spans="1:24">
       <c r="A9">
         <v>7</v>
       </c>
@@ -4247,7 +3630,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="10" spans="1:22">
+    <row r="10" spans="1:24">
       <c r="A10">
         <v>8</v>
       </c>
@@ -4309,7 +3692,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="11" spans="1:22">
+    <row r="11" spans="1:24">
       <c r="A11">
         <v>9</v>
       </c>
@@ -4371,7 +3754,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="12" spans="1:22">
+    <row r="12" spans="1:24">
       <c r="A12">
         <v>10</v>
       </c>
@@ -4433,7 +3816,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="13" ht="15.95" customHeight="1" spans="1:22">
+    <row r="13" spans="1:24" ht="15.95" customHeight="1">
       <c r="A13">
         <v>11</v>
       </c>
@@ -4495,7 +3878,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="14" spans="1:22">
+    <row r="14" spans="1:24">
       <c r="A14">
         <v>12</v>
       </c>
@@ -4557,7 +3940,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="15" spans="1:22">
+    <row r="15" spans="1:24">
       <c r="A15">
         <v>13</v>
       </c>
@@ -4619,7 +4002,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="16" spans="1:23">
+    <row r="16" spans="1:24">
       <c r="A16">
         <v>14</v>
       </c>
@@ -4684,7 +4067,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="17" spans="1:22">
+    <row r="17" spans="1:23">
       <c r="A17">
         <v>15</v>
       </c>
@@ -4746,7 +4129,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="18" spans="1:22">
+    <row r="18" spans="1:23">
       <c r="A18">
         <v>16</v>
       </c>
@@ -4808,7 +4191,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="19" spans="1:22">
+    <row r="19" spans="1:23">
       <c r="A19">
         <v>17</v>
       </c>
@@ -5000,7 +4383,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="22" spans="1:21">
+    <row r="22" spans="1:23">
       <c r="A22">
         <v>20</v>
       </c>
@@ -5059,7 +4442,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="23" spans="1:21">
+    <row r="23" spans="1:23">
       <c r="A23">
         <v>21</v>
       </c>
@@ -5118,47 +4501,45 @@
         <v>140</v>
       </c>
     </row>
-    <row r="24" spans="19:19">
+    <row r="24" spans="1:23">
       <c r="S24" s="2"/>
     </row>
-    <row r="25" spans="19:19">
+    <row r="25" spans="1:23">
       <c r="S25" s="2"/>
     </row>
-    <row r="26" spans="19:19">
+    <row r="26" spans="1:23">
       <c r="S26" s="2"/>
     </row>
-    <row r="27" spans="19:19">
+    <row r="27" spans="1:23">
       <c r="S27" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:V75"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="10.4259259259259" style="2" customWidth="1"/>
-    <col min="2" max="2" width="23.287037037037" style="2" customWidth="1"/>
-    <col min="3" max="3" width="27.712962962963" style="2" customWidth="1"/>
-    <col min="4" max="4" width="10.1388888888889" style="2" customWidth="1"/>
-    <col min="5" max="5" width="8.13888888888889" style="2" customWidth="1"/>
-    <col min="6" max="6" width="8.42592592592593" style="2" customWidth="1"/>
-    <col min="7" max="7" width="6.85185185185185" style="2" customWidth="1"/>
-    <col min="8" max="8" width="10.287037037037" style="2" customWidth="1"/>
-    <col min="9" max="9" width="15.5740740740741" style="2" customWidth="1"/>
-    <col min="10" max="10" width="16.8518518518519" style="2" customWidth="1"/>
-    <col min="11" max="11" width="19.287037037037" style="2" customWidth="1"/>
-    <col min="12" max="12" width="16.8518518518519" style="2" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="6.85546875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="10.28515625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" style="2" customWidth="1"/>
+    <col min="10" max="10" width="16.85546875" style="2" customWidth="1"/>
+    <col min="11" max="11" width="19.28515625" style="2" customWidth="1"/>
+    <col min="12" max="12" width="16.85546875" style="2" customWidth="1"/>
     <col min="13" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:22">
+    <row r="1" spans="1:22" ht="30" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -5226,7 +4607,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="2" customHeight="1" spans="1:14">
+    <row r="2" spans="1:22" ht="30" customHeight="1">
       <c r="A2" s="2">
         <v>0</v>
       </c>
@@ -5264,7 +4645,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" customHeight="1" spans="1:14">
+    <row r="3" spans="1:22" ht="30" customHeight="1">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -5302,7 +4683,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" customHeight="1" spans="1:14">
+    <row r="4" spans="1:22" ht="30" customHeight="1">
       <c r="A4" s="2">
         <v>2</v>
       </c>
@@ -5340,7 +4721,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" customHeight="1" spans="1:14">
+    <row r="5" spans="1:22" ht="30" customHeight="1">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -5375,7 +4756,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" ht="33" customHeight="1" spans="1:15">
+    <row r="6" spans="1:22" ht="33" customHeight="1">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -5413,7 +4794,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" customHeight="1" spans="1:16">
+    <row r="7" spans="1:22" ht="30" customHeight="1">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -5454,7 +4835,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="8" customHeight="1" spans="1:12">
+    <row r="8" spans="1:22" ht="30" customHeight="1">
       <c r="A8" s="2">
         <v>6</v>
       </c>
@@ -5486,7 +4867,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="9" customHeight="1" spans="1:12">
+    <row r="9" spans="1:22" ht="30" customHeight="1">
       <c r="A9" s="2">
         <v>7</v>
       </c>
@@ -5518,7 +4899,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="10" customHeight="1" spans="1:12">
+    <row r="10" spans="1:22" ht="30" customHeight="1">
       <c r="A10" s="2">
         <v>8</v>
       </c>
@@ -5550,7 +4931,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="11" customHeight="1" spans="1:12">
+    <row r="11" spans="1:22" ht="30" customHeight="1">
       <c r="A11" s="2">
         <v>9</v>
       </c>
@@ -5582,7 +4963,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="12" customHeight="1" spans="1:12">
+    <row r="12" spans="1:22" ht="30" customHeight="1">
       <c r="A12" s="2">
         <v>10</v>
       </c>
@@ -5614,7 +4995,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="13" customHeight="1" spans="1:12">
+    <row r="13" spans="1:22" ht="30" customHeight="1">
       <c r="A13" s="2">
         <v>11</v>
       </c>
@@ -5646,7 +5027,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="14" customHeight="1" spans="1:12">
+    <row r="14" spans="1:22" ht="30" customHeight="1">
       <c r="A14" s="2">
         <v>12</v>
       </c>
@@ -5681,7 +5062,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="15" customHeight="1" spans="1:12">
+    <row r="15" spans="1:22" ht="30" customHeight="1">
       <c r="A15" s="2">
         <v>13</v>
       </c>
@@ -5716,7 +5097,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="16" ht="42" customHeight="1" spans="1:12">
+    <row r="16" spans="1:22" ht="42" customHeight="1">
       <c r="A16" s="2">
         <v>14</v>
       </c>
@@ -5746,7 +5127,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="17" customHeight="1" spans="1:12">
+    <row r="17" spans="1:12" ht="30" customHeight="1">
       <c r="A17" s="2">
         <v>15</v>
       </c>
@@ -5776,7 +5157,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="18" customHeight="1" spans="1:12">
+    <row r="18" spans="1:12" ht="30" customHeight="1">
       <c r="A18" s="2">
         <v>16</v>
       </c>
@@ -5806,7 +5187,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="19" customHeight="1" spans="1:12">
+    <row r="19" spans="1:12" ht="30" customHeight="1">
       <c r="A19" s="2">
         <v>17</v>
       </c>
@@ -5838,7 +5219,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="20" customHeight="1" spans="1:12">
+    <row r="20" spans="1:12" ht="30" customHeight="1">
       <c r="A20" s="2">
         <v>18</v>
       </c>
@@ -5870,7 +5251,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="21" customHeight="1" spans="1:12">
+    <row r="21" spans="1:12" ht="30" customHeight="1">
       <c r="A21" s="2">
         <v>19</v>
       </c>
@@ -5902,7 +5283,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="22" customHeight="1" spans="1:12">
+    <row r="22" spans="1:12" ht="30" customHeight="1">
       <c r="A22" s="2">
         <v>20</v>
       </c>
@@ -5934,7 +5315,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="23" customHeight="1" spans="1:12">
+    <row r="23" spans="1:12" ht="30" customHeight="1">
       <c r="A23" s="2">
         <v>21</v>
       </c>
@@ -5966,7 +5347,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="24" customHeight="1" spans="1:12">
+    <row r="24" spans="1:12" ht="30" customHeight="1">
       <c r="A24" s="2">
         <v>22</v>
       </c>
@@ -5998,7 +5379,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="25" customHeight="1" spans="1:12">
+    <row r="25" spans="1:12" ht="30" customHeight="1">
       <c r="A25" s="2">
         <v>23</v>
       </c>
@@ -6030,7 +5411,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="26" customHeight="1" spans="1:12">
+    <row r="26" spans="1:12" ht="30" customHeight="1">
       <c r="A26" s="2">
         <v>24</v>
       </c>
@@ -6062,7 +5443,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="27" customHeight="1" spans="1:12">
+    <row r="27" spans="1:12" ht="30" customHeight="1">
       <c r="A27" s="2">
         <v>25</v>
       </c>
@@ -6094,7 +5475,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="28" customHeight="1" spans="1:12">
+    <row r="28" spans="1:12" ht="30" customHeight="1">
       <c r="A28" s="2">
         <v>26</v>
       </c>
@@ -6126,7 +5507,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="29" customHeight="1" spans="1:12">
+    <row r="29" spans="1:12" ht="30" customHeight="1">
       <c r="A29" s="2">
         <v>27</v>
       </c>
@@ -6158,7 +5539,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="30" customHeight="1" spans="1:12">
+    <row r="30" spans="1:12" ht="30" customHeight="1">
       <c r="A30" s="2">
         <v>28</v>
       </c>
@@ -6190,7 +5571,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="31" customHeight="1" spans="1:9">
+    <row r="31" spans="1:12" ht="30" customHeight="1">
       <c r="A31" s="2">
         <v>29</v>
       </c>
@@ -6219,7 +5600,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="32" customHeight="1" spans="1:12">
+    <row r="32" spans="1:12" ht="30" customHeight="1">
       <c r="A32" s="2">
         <v>30</v>
       </c>
@@ -6251,7 +5632,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="33" customHeight="1" spans="1:12">
+    <row r="33" spans="1:12" ht="30" customHeight="1">
       <c r="A33" s="2">
         <v>31</v>
       </c>
@@ -6283,7 +5664,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="34" customHeight="1" spans="1:12">
+    <row r="34" spans="1:12" ht="30" customHeight="1">
       <c r="A34" s="2">
         <v>32</v>
       </c>
@@ -6315,7 +5696,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="35" customHeight="1" spans="1:12">
+    <row r="35" spans="1:12" ht="30" customHeight="1">
       <c r="A35" s="2">
         <v>33</v>
       </c>
@@ -6347,7 +5728,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="36" customHeight="1" spans="1:12">
+    <row r="36" spans="1:12" ht="30" customHeight="1">
       <c r="A36" s="2">
         <v>34</v>
       </c>
@@ -6379,7 +5760,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="37" customHeight="1" spans="1:12">
+    <row r="37" spans="1:12" ht="30" customHeight="1">
       <c r="A37" s="2">
         <v>35</v>
       </c>
@@ -6411,7 +5792,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="38" customHeight="1" spans="1:12">
+    <row r="38" spans="1:12" ht="30" customHeight="1">
       <c r="A38" s="2">
         <v>36</v>
       </c>
@@ -6443,7 +5824,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="39" customHeight="1" spans="1:12">
+    <row r="39" spans="1:12" ht="30" customHeight="1">
       <c r="A39" s="2">
         <v>37</v>
       </c>
@@ -6475,7 +5856,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="40" customHeight="1" spans="1:12">
+    <row r="40" spans="1:12" ht="30" customHeight="1">
       <c r="A40" s="2">
         <v>38</v>
       </c>
@@ -6507,7 +5888,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="41" customHeight="1" spans="1:12">
+    <row r="41" spans="1:12" ht="30" customHeight="1">
       <c r="A41" s="2">
         <v>39</v>
       </c>
@@ -6539,7 +5920,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="42" customHeight="1" spans="1:12">
+    <row r="42" spans="1:12" ht="30" customHeight="1">
       <c r="A42" s="2">
         <v>40</v>
       </c>
@@ -6571,7 +5952,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="43" customHeight="1" spans="1:12">
+    <row r="43" spans="1:12" ht="30" customHeight="1">
       <c r="A43" s="2">
         <v>41</v>
       </c>
@@ -6603,7 +5984,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="44" customHeight="1" spans="1:12">
+    <row r="44" spans="1:12" ht="30" customHeight="1">
       <c r="A44" s="2">
         <v>42</v>
       </c>
@@ -6635,7 +6016,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="45" customHeight="1" spans="1:12">
+    <row r="45" spans="1:12" ht="30" customHeight="1">
       <c r="A45" s="2">
         <v>43</v>
       </c>
@@ -6667,7 +6048,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="46" customHeight="1" spans="1:12">
+    <row r="46" spans="1:12" ht="30" customHeight="1">
       <c r="A46" s="2">
         <v>44</v>
       </c>
@@ -6699,7 +6080,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="47" customHeight="1" spans="1:12">
+    <row r="47" spans="1:12" ht="30" customHeight="1">
       <c r="A47" s="2">
         <v>45</v>
       </c>
@@ -6731,7 +6112,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="48" customHeight="1" spans="1:12">
+    <row r="48" spans="1:12" ht="30" customHeight="1">
       <c r="A48" s="2">
         <v>46</v>
       </c>
@@ -6763,7 +6144,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="49" customHeight="1" spans="1:12">
+    <row r="49" spans="1:12" ht="30" customHeight="1">
       <c r="A49" s="2">
         <v>47</v>
       </c>
@@ -6795,7 +6176,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="50" customHeight="1" spans="1:12">
+    <row r="50" spans="1:12" ht="30" customHeight="1">
       <c r="A50" s="2">
         <v>48</v>
       </c>
@@ -6830,7 +6211,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="51" customHeight="1" spans="1:12">
+    <row r="51" spans="1:12" ht="30" customHeight="1">
       <c r="A51" s="2">
         <v>49</v>
       </c>
@@ -6865,7 +6246,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="52" customHeight="1" spans="1:12">
+    <row r="52" spans="1:12" ht="30" customHeight="1">
       <c r="A52" s="2">
         <v>50</v>
       </c>
@@ -6900,7 +6281,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="53" customHeight="1" spans="1:12">
+    <row r="53" spans="1:12" ht="30" customHeight="1">
       <c r="A53" s="2">
         <v>51</v>
       </c>
@@ -6935,7 +6316,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="54" customHeight="1" spans="1:12">
+    <row r="54" spans="1:12" ht="30" customHeight="1">
       <c r="A54" s="2">
         <v>52</v>
       </c>
@@ -6970,7 +6351,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="55" ht="124.2" spans="1:12">
+    <row r="55" spans="1:12" ht="165">
       <c r="A55" s="2">
         <v>53</v>
       </c>
@@ -7002,7 +6383,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="56" ht="124.2" spans="1:12">
+    <row r="56" spans="1:12" ht="165">
       <c r="A56" s="2">
         <v>54</v>
       </c>
@@ -7034,7 +6415,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="57" ht="110.4" spans="1:12">
+    <row r="57" spans="1:12" ht="135">
       <c r="A57" s="2">
         <v>55</v>
       </c>
@@ -7066,7 +6447,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="58" ht="110.4" spans="1:12">
+    <row r="58" spans="1:12" ht="135">
       <c r="A58" s="2">
         <v>56</v>
       </c>
@@ -7098,7 +6479,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="59" ht="110.4" spans="1:12">
+    <row r="59" spans="1:12" ht="135">
       <c r="A59" s="2">
         <v>57</v>
       </c>
@@ -7130,7 +6511,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="60" ht="110.4" spans="1:12">
+    <row r="60" spans="1:12" ht="135">
       <c r="A60" s="2">
         <v>58</v>
       </c>
@@ -7162,7 +6543,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="61" ht="110.4" spans="1:12">
+    <row r="61" spans="1:12" ht="135">
       <c r="A61" s="2">
         <v>59</v>
       </c>
@@ -7194,7 +6575,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="62" ht="96.6" spans="1:12">
+    <row r="62" spans="1:12" ht="120">
       <c r="A62" s="2">
         <v>60</v>
       </c>
@@ -7226,7 +6607,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="63" ht="96.6" spans="1:12">
+    <row r="63" spans="1:12" ht="120">
       <c r="A63" s="2">
         <v>61</v>
       </c>
@@ -7258,7 +6639,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="64" ht="96.6" spans="1:12">
+    <row r="64" spans="1:12" ht="120">
       <c r="A64" s="2">
         <v>62</v>
       </c>
@@ -7290,7 +6671,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="65" ht="96.6" spans="1:12">
+    <row r="65" spans="1:12" ht="120">
       <c r="A65" s="2">
         <v>63</v>
       </c>
@@ -7322,7 +6703,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="66" ht="13.8" spans="1:12">
+    <row r="66" spans="1:12" ht="15">
       <c r="A66" s="2">
         <v>64</v>
       </c>
@@ -7354,7 +6735,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="67" ht="13.8" spans="1:12">
+    <row r="67" spans="1:12" ht="15">
       <c r="A67" s="2">
         <v>65</v>
       </c>
@@ -7386,7 +6767,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="68" ht="13.8" spans="1:12">
+    <row r="68" spans="1:12" ht="15">
       <c r="A68" s="2">
         <v>66</v>
       </c>
@@ -7418,7 +6799,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="69" ht="13.8" spans="1:12">
+    <row r="69" spans="1:12" ht="15">
       <c r="A69" s="2">
         <v>67</v>
       </c>
@@ -7450,7 +6831,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="70" ht="13.8" spans="1:12">
+    <row r="70" spans="1:12" ht="15">
       <c r="A70" s="2">
         <v>68</v>
       </c>
@@ -7482,7 +6863,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="71" ht="13.8" spans="1:12">
+    <row r="71" spans="1:12" ht="15">
       <c r="A71" s="2">
         <v>69</v>
       </c>
@@ -7514,7 +6895,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="72" ht="13.8" spans="1:12">
+    <row r="72" spans="1:12" ht="15">
       <c r="A72" s="2">
         <v>70</v>
       </c>
@@ -7546,7 +6927,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="73" ht="13.8" spans="1:12">
+    <row r="73" spans="1:12" ht="15">
       <c r="A73" s="2">
         <v>71</v>
       </c>
@@ -7575,7 +6956,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="74" ht="41.4" spans="1:9">
+    <row r="74" spans="1:12" ht="45">
       <c r="A74" s="2">
         <v>72</v>
       </c>
@@ -7604,24 +6985,22 @@
         <v>447</v>
       </c>
     </row>
-    <row r="75" ht="13.8"/>
+    <row r="75" spans="1:12" ht="15"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="17.287037037037" customWidth="1"/>
-    <col min="4" max="4" width="20.1388888888889" customWidth="1"/>
-    <col min="5" max="5" width="19.712962962963" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" customWidth="1"/>
+    <col min="5" max="5" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -7783,21 +7162,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="13.8" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.66666666666667" customWidth="1"/>
-    <col min="2" max="2" width="18.6666666666667" customWidth="1"/>
-    <col min="3" max="3" width="11.4444444444444" customWidth="1"/>
-    <col min="4" max="4" width="28.8888888888889" customWidth="1"/>
-    <col min="5" max="5" width="12.7777777777778" customWidth="1"/>
+    <col min="1" max="1" width="3.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="28.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -7959,25 +7336,23 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:M9"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:N9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.4259259259259" customWidth="1"/>
-    <col min="2" max="2" width="15.1388888888889" customWidth="1"/>
-    <col min="3" max="3" width="20.287037037037" customWidth="1"/>
-    <col min="4" max="4" width="16.8518518518519" customWidth="1"/>
-    <col min="6" max="6" width="10.712962962963" customWidth="1"/>
-    <col min="7" max="7" width="11.287037037037" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" customWidth="1"/>
+    <col min="3" max="3" width="20.28515625" customWidth="1"/>
+    <col min="4" max="5" width="16.85546875" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -7991,126 +7366,141 @@
         <v>127</v>
       </c>
       <c r="E1" t="s">
+        <v>504</v>
+      </c>
+      <c r="F1" t="s">
         <v>483</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>484</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>485</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>228</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>230</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:14">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2" t="s">
         <v>486</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
         <v>487</v>
       </c>
-      <c r="F2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G2">
+      <c r="G2" t="s">
         <v>0</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:14">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>488</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" t="s">
         <v>487</v>
       </c>
-      <c r="F3" t="s">
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
+      <c r="G3" t="s">
+        <v>0</v>
       </c>
       <c r="H3">
         <v>1</v>
       </c>
       <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:14">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
         <v>489</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="s">
         <v>487</v>
       </c>
-      <c r="F4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>2</v>
+      <c r="G4" t="s">
+        <v>0</v>
       </c>
       <c r="H4">
         <v>2</v>
       </c>
       <c r="I4">
+        <v>2</v>
+      </c>
+      <c r="J4">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:14">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" t="s">
         <v>490</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="s">
         <v>491</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>492</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>279</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>5</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:14">
       <c r="A6">
         <v>4</v>
       </c>
@@ -8120,23 +7510,26 @@
       <c r="C6" t="s">
         <v>494</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6" t="s">
         <v>487</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>495</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>12</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>15</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:14">
       <c r="A7">
         <v>5</v>
       </c>
@@ -8146,20 +7539,23 @@
       <c r="C7" t="s">
         <v>497</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7" t="s">
         <v>498</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>3</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>144</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:14">
       <c r="A8">
         <v>6</v>
       </c>
@@ -8169,20 +7565,23 @@
       <c r="C8" t="s">
         <v>500</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8" t="s">
         <v>487</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>3</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>311</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:14">
       <c r="A9">
         <v>7</v>
       </c>
@@ -8192,25 +7591,27 @@
       <c r="C9" t="s">
         <v>502</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9" t="s">
         <v>503</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>3</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>144</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>15</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <v>30</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finished Raising Animation System
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Raising.xlsx
+++ b/Assets/StreamingAssets/Configurations/Raising.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9DB62DB-5781-4004-915C-10D028310E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A66741A5-6ACD-4E73-9CE1-91A8618687CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingEffects" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1052" uniqueCount="505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="508">
   <si>
     <t>ID</t>
   </si>
@@ -1579,6 +1579,15 @@
   </si>
   <si>
     <t>在事件前执行</t>
+  </si>
+  <si>
+    <t>0.2,0.7,0.1,0.8,0.2,0.1</t>
+  </si>
+  <si>
+    <t>VRaisingReplaceCardEffect</t>
+  </si>
+  <si>
+    <t>replace card</t>
   </si>
 </sst>
 </file>
@@ -2017,7 +2026,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.42578125" customWidth="1"/>
@@ -3029,6 +3038,20 @@
       </c>
       <c r="F66" t="s">
         <v>81</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6">
+      <c r="A67">
+        <v>65</v>
+      </c>
+      <c r="B67" t="s">
+        <v>507</v>
+      </c>
+      <c r="D67" t="s">
+        <v>506</v>
+      </c>
+      <c r="F67" t="s">
+        <v>505</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed audio, added new scheduling condition pattern
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Raising.xlsx
+++ b/Assets/StreamingAssets/Configurations/Raising.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F7C4C43-119A-486E-8C1B-7E358AF4270E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="10030" activeTab="2"/>
+    <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingEffects" sheetId="1" r:id="rId1"/>
@@ -26,8 +32,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -1703,18 +1707,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="21">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -1724,152 +1722,8 @@
       <name val="宋体"/>
       <charset val="134"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="43">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1908,7 +1762,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.0999786370433668"/>
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1936,194 +1790,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -2140,251 +1808,9 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="15" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -2438,75 +1864,31 @@
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="00DEBA2C"/>
-      <color rgb="00FD460D"/>
-      <color rgb="00A122FB"/>
-      <color rgb="004C8BFE"/>
-      <color rgb="004058E8"/>
-      <color rgb="0057CDD2"/>
-      <color rgb="0052F620"/>
-      <color rgb="000FEFDD"/>
-      <color rgb="0010CCEE"/>
-      <color rgb="008AE72F"/>
+      <color rgb="FFDEBA2C"/>
+      <color rgb="FFFD460D"/>
+      <color rgb="FFA122FB"/>
+      <color rgb="FF4C8BFE"/>
+      <color rgb="FF4058E8"/>
+      <color rgb="FF57CDD2"/>
+      <color rgb="FF52F620"/>
+      <color rgb="FF0FEFDD"/>
+      <color rgb="FF10CCEE"/>
+      <color rgb="FF8AE72F"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -2764,22 +2146,22 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F68"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.425" customWidth="1"/>
-    <col min="2" max="2" width="31.425" customWidth="1"/>
-    <col min="3" max="3" width="29.425" customWidth="1"/>
-    <col min="4" max="4" width="31.7166666666667" customWidth="1"/>
-    <col min="5" max="5" width="15.2833333333333" customWidth="1"/>
-    <col min="6" max="6" width="29.575" customWidth="1"/>
-    <col min="7" max="7" width="15.7166666666667" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="31.42578125" customWidth="1"/>
+    <col min="3" max="3" width="29.42578125" customWidth="1"/>
+    <col min="4" max="4" width="31.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" customWidth="1"/>
+    <col min="6" max="6" width="29.5703125" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -3811,36 +3193,34 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:X27"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.425" customWidth="1"/>
-    <col min="2" max="2" width="21.85" customWidth="1"/>
-    <col min="3" max="3" width="22.2833333333333" customWidth="1"/>
-    <col min="4" max="4" width="11.575" customWidth="1"/>
-    <col min="5" max="6" width="11.425" customWidth="1"/>
-    <col min="7" max="7" width="6.71666666666667" customWidth="1"/>
-    <col min="9" max="9" width="8.14166666666667" customWidth="1"/>
-    <col min="10" max="11" width="15.425" customWidth="1"/>
-    <col min="12" max="12" width="10.7166666666667" customWidth="1"/>
-    <col min="13" max="13" width="3.28333333333333" customWidth="1"/>
-    <col min="14" max="14" width="6.425" customWidth="1"/>
-    <col min="15" max="15" width="11.7166666666667" customWidth="1"/>
-    <col min="16" max="16" width="10.2833333333333" customWidth="1"/>
-    <col min="17" max="17" width="10.7166666666667" customWidth="1"/>
-    <col min="18" max="18" width="11.85" customWidth="1"/>
-    <col min="19" max="19" width="8.28333333333333" customWidth="1"/>
-    <col min="20" max="20" width="10.1416666666667" customWidth="1"/>
-    <col min="21" max="21" width="14.1416666666667" customWidth="1"/>
-    <col min="22" max="22" width="10.2833333333333" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" customWidth="1"/>
+    <col min="3" max="3" width="22.28515625" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" customWidth="1"/>
+    <col min="5" max="6" width="11.42578125" customWidth="1"/>
+    <col min="7" max="7" width="6.7109375" customWidth="1"/>
+    <col min="9" max="9" width="8.140625" customWidth="1"/>
+    <col min="10" max="11" width="15.42578125" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" customWidth="1"/>
+    <col min="13" max="13" width="3.28515625" customWidth="1"/>
+    <col min="14" max="14" width="6.42578125" customWidth="1"/>
+    <col min="15" max="15" width="11.7109375" customWidth="1"/>
+    <col min="16" max="16" width="10.28515625" customWidth="1"/>
+    <col min="17" max="17" width="10.7109375" customWidth="1"/>
+    <col min="18" max="18" width="11.85546875" customWidth="1"/>
+    <col min="19" max="19" width="8.28515625" customWidth="1"/>
+    <col min="20" max="20" width="10.140625" customWidth="1"/>
+    <col min="21" max="21" width="14.140625" customWidth="1"/>
+    <col min="22" max="22" width="10.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24">
@@ -3917,7 +3297,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="2" ht="42" spans="1:24">
+    <row r="2" spans="1:24" ht="60">
       <c r="A2">
         <v>0</v>
       </c>
@@ -3979,7 +3359,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" ht="42" spans="1:24">
+    <row r="3" spans="1:24" ht="60">
       <c r="A3">
         <v>1</v>
       </c>
@@ -4041,7 +3421,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" ht="42" spans="1:24">
+    <row r="4" spans="1:24" ht="60">
       <c r="A4">
         <v>2</v>
       </c>
@@ -4596,7 +3976,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="13" ht="15.95" customHeight="1" spans="1:24">
+    <row r="13" spans="1:24" ht="15.95" customHeight="1">
       <c r="A13">
         <v>11</v>
       </c>
@@ -5407,33 +4787,31 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:V84"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="10.425" style="2" customWidth="1"/>
-    <col min="2" max="2" width="23.2833333333333" style="2" customWidth="1"/>
-    <col min="3" max="3" width="37.5833333333333" style="2" customWidth="1"/>
-    <col min="4" max="4" width="10.1416666666667" style="2" customWidth="1"/>
-    <col min="5" max="5" width="8.14166666666667" style="2" customWidth="1"/>
-    <col min="6" max="6" width="8.425" style="2" customWidth="1"/>
-    <col min="7" max="7" width="6.85" style="2" customWidth="1"/>
-    <col min="8" max="8" width="10.2833333333333" style="2" customWidth="1"/>
-    <col min="9" max="9" width="15.575" style="2" customWidth="1"/>
-    <col min="10" max="10" width="16.85" style="2" customWidth="1"/>
-    <col min="11" max="11" width="19.2833333333333" style="2" customWidth="1"/>
-    <col min="12" max="12" width="16.85" style="2" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="37.5703125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="6.85546875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="10.28515625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" style="2" customWidth="1"/>
+    <col min="10" max="10" width="16.85546875" style="2" customWidth="1"/>
+    <col min="11" max="11" width="19.28515625" style="2" customWidth="1"/>
+    <col min="12" max="12" width="16.85546875" style="2" customWidth="1"/>
     <col min="13" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:22">
+    <row r="1" spans="1:22" ht="30" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -5501,7 +4879,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="2" customHeight="1" spans="1:22">
+    <row r="2" spans="1:22" ht="30" customHeight="1">
       <c r="A2" s="2">
         <v>0</v>
       </c>
@@ -5539,7 +4917,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" customHeight="1" spans="1:22">
+    <row r="3" spans="1:22" ht="30" customHeight="1">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -5577,7 +4955,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" customHeight="1" spans="1:22">
+    <row r="4" spans="1:22" ht="30" customHeight="1">
       <c r="A4" s="2">
         <v>2</v>
       </c>
@@ -5615,7 +4993,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" customHeight="1" spans="1:22">
+    <row r="5" spans="1:22" ht="30" customHeight="1">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -5650,7 +5028,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" ht="33" customHeight="1" spans="1:22">
+    <row r="6" spans="1:22" ht="33" customHeight="1">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -5688,7 +5066,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" customHeight="1" spans="1:22">
+    <row r="7" spans="1:22" ht="30" customHeight="1">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -5729,7 +5107,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="8" customHeight="1" spans="1:22">
+    <row r="8" spans="1:22" ht="30" customHeight="1">
       <c r="A8" s="2">
         <v>6</v>
       </c>
@@ -5761,7 +5139,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="9" customHeight="1" spans="1:22">
+    <row r="9" spans="1:22" ht="30" customHeight="1">
       <c r="A9" s="2">
         <v>7</v>
       </c>
@@ -5793,7 +5171,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="10" customHeight="1" spans="1:22">
+    <row r="10" spans="1:22" ht="30" customHeight="1">
       <c r="A10" s="2">
         <v>8</v>
       </c>
@@ -5825,7 +5203,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="11" customHeight="1" spans="1:22">
+    <row r="11" spans="1:22" ht="30" customHeight="1">
       <c r="A11" s="2">
         <v>9</v>
       </c>
@@ -5857,7 +5235,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="12" customHeight="1" spans="1:22">
+    <row r="12" spans="1:22" ht="30" customHeight="1">
       <c r="A12" s="2">
         <v>10</v>
       </c>
@@ -5889,7 +5267,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="13" customHeight="1" spans="1:22">
+    <row r="13" spans="1:22" ht="30" customHeight="1">
       <c r="A13" s="2">
         <v>11</v>
       </c>
@@ -5924,7 +5302,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="14" customHeight="1" spans="1:22">
+    <row r="14" spans="1:22" ht="30" customHeight="1">
       <c r="A14" s="2">
         <v>12</v>
       </c>
@@ -5959,7 +5337,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="15" customHeight="1" spans="1:22">
+    <row r="15" spans="1:22" ht="30" customHeight="1">
       <c r="A15" s="2">
         <v>13</v>
       </c>
@@ -5994,7 +5372,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="16" ht="42" customHeight="1" spans="1:22">
+    <row r="16" spans="1:22" ht="42" customHeight="1">
       <c r="A16" s="2">
         <v>14</v>
       </c>
@@ -6024,7 +5402,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="17" customHeight="1" spans="1:14">
+    <row r="17" spans="1:14" ht="30" customHeight="1">
       <c r="A17" s="2">
         <v>15</v>
       </c>
@@ -6054,7 +5432,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="18" customHeight="1" spans="1:14">
+    <row r="18" spans="1:14" ht="30" customHeight="1">
       <c r="A18" s="2">
         <v>16</v>
       </c>
@@ -6084,7 +5462,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="19" customHeight="1" spans="1:14">
+    <row r="19" spans="1:14" ht="30" customHeight="1">
       <c r="A19" s="2">
         <v>17</v>
       </c>
@@ -6116,7 +5494,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="20" customHeight="1" spans="1:14">
+    <row r="20" spans="1:14" ht="30" customHeight="1">
       <c r="A20" s="2">
         <v>18</v>
       </c>
@@ -6148,7 +5526,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="21" customHeight="1" spans="1:14">
+    <row r="21" spans="1:14" ht="30" customHeight="1">
       <c r="A21" s="2">
         <v>19</v>
       </c>
@@ -6180,7 +5558,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="22" customHeight="1" spans="1:14">
+    <row r="22" spans="1:14" ht="30" customHeight="1">
       <c r="A22" s="2">
         <v>20</v>
       </c>
@@ -6212,7 +5590,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="23" customHeight="1" spans="1:14">
+    <row r="23" spans="1:14" ht="30" customHeight="1">
       <c r="A23" s="2">
         <v>21</v>
       </c>
@@ -6244,7 +5622,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="24" customHeight="1" spans="1:14">
+    <row r="24" spans="1:14" ht="30" customHeight="1">
       <c r="A24" s="2">
         <v>22</v>
       </c>
@@ -6276,7 +5654,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="25" customHeight="1" spans="1:14">
+    <row r="25" spans="1:14" ht="30" customHeight="1">
       <c r="A25" s="2">
         <v>23</v>
       </c>
@@ -6308,7 +5686,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="26" customHeight="1" spans="1:14">
+    <row r="26" spans="1:14" ht="30" customHeight="1">
       <c r="A26" s="2">
         <v>24</v>
       </c>
@@ -6343,7 +5721,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" customHeight="1" spans="1:14">
+    <row r="27" spans="1:14" ht="30" customHeight="1">
       <c r="A27" s="2">
         <v>25</v>
       </c>
@@ -6378,7 +5756,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" customHeight="1" spans="1:14">
+    <row r="28" spans="1:14" ht="30" customHeight="1">
       <c r="A28" s="2">
         <v>26</v>
       </c>
@@ -6413,7 +5791,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" customHeight="1" spans="1:14">
+    <row r="29" spans="1:14" ht="30" customHeight="1">
       <c r="A29" s="2">
         <v>27</v>
       </c>
@@ -6448,7 +5826,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" customHeight="1" spans="1:14">
+    <row r="30" spans="1:14" ht="30" customHeight="1">
       <c r="A30" s="2">
         <v>28</v>
       </c>
@@ -6483,7 +5861,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" customHeight="1" spans="1:14">
+    <row r="31" spans="1:14" ht="30" customHeight="1">
       <c r="A31" s="2">
         <v>29</v>
       </c>
@@ -6512,7 +5890,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="32" customHeight="1" spans="1:14">
+    <row r="32" spans="1:14" ht="30" customHeight="1">
       <c r="A32" s="2">
         <v>30</v>
       </c>
@@ -6544,7 +5922,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="33" customHeight="1" spans="1:12">
+    <row r="33" spans="1:12" ht="30" customHeight="1">
       <c r="A33" s="2">
         <v>31</v>
       </c>
@@ -6576,7 +5954,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="34" customHeight="1" spans="1:12">
+    <row r="34" spans="1:12" ht="30" customHeight="1">
       <c r="A34" s="2">
         <v>32</v>
       </c>
@@ -6608,7 +5986,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="35" customHeight="1" spans="1:12">
+    <row r="35" spans="1:12" ht="30" customHeight="1">
       <c r="A35" s="2">
         <v>33</v>
       </c>
@@ -6640,7 +6018,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="36" customHeight="1" spans="1:12">
+    <row r="36" spans="1:12" ht="30" customHeight="1">
       <c r="A36" s="2">
         <v>34</v>
       </c>
@@ -6672,7 +6050,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="37" customHeight="1" spans="1:12">
+    <row r="37" spans="1:12" ht="30" customHeight="1">
       <c r="A37" s="2">
         <v>35</v>
       </c>
@@ -6704,7 +6082,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="38" customHeight="1" spans="1:12">
+    <row r="38" spans="1:12" ht="30" customHeight="1">
       <c r="A38" s="2">
         <v>36</v>
       </c>
@@ -6736,7 +6114,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="39" customHeight="1" spans="1:12">
+    <row r="39" spans="1:12" ht="30" customHeight="1">
       <c r="A39" s="2">
         <v>37</v>
       </c>
@@ -6768,7 +6146,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="40" customHeight="1" spans="1:12">
+    <row r="40" spans="1:12" ht="30" customHeight="1">
       <c r="A40" s="2">
         <v>38</v>
       </c>
@@ -6800,7 +6178,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="41" customHeight="1" spans="1:12">
+    <row r="41" spans="1:12" ht="30" customHeight="1">
       <c r="A41" s="2">
         <v>39</v>
       </c>
@@ -6832,7 +6210,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="42" customHeight="1" spans="1:12">
+    <row r="42" spans="1:12" ht="30" customHeight="1">
       <c r="A42" s="2">
         <v>40</v>
       </c>
@@ -6864,7 +6242,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="43" customHeight="1" spans="1:12">
+    <row r="43" spans="1:12" ht="30" customHeight="1">
       <c r="A43" s="2">
         <v>41</v>
       </c>
@@ -6896,7 +6274,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="44" customHeight="1" spans="1:12">
+    <row r="44" spans="1:12" ht="30" customHeight="1">
       <c r="A44" s="2">
         <v>42</v>
       </c>
@@ -6928,7 +6306,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="45" customHeight="1" spans="1:12">
+    <row r="45" spans="1:12" ht="30" customHeight="1">
       <c r="A45" s="2">
         <v>43</v>
       </c>
@@ -6960,7 +6338,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="46" customHeight="1" spans="1:12">
+    <row r="46" spans="1:12" ht="30" customHeight="1">
       <c r="A46" s="2">
         <v>44</v>
       </c>
@@ -6992,7 +6370,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="47" customHeight="1" spans="1:12">
+    <row r="47" spans="1:12" ht="30" customHeight="1">
       <c r="A47" s="2">
         <v>45</v>
       </c>
@@ -7024,7 +6402,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="48" customHeight="1" spans="1:12">
+    <row r="48" spans="1:12" ht="30" customHeight="1">
       <c r="A48" s="2">
         <v>46</v>
       </c>
@@ -7056,7 +6434,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="49" customHeight="1" spans="1:12">
+    <row r="49" spans="1:12" ht="30" customHeight="1">
       <c r="A49" s="2">
         <v>47</v>
       </c>
@@ -7088,7 +6466,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="50" customHeight="1" spans="1:12">
+    <row r="50" spans="1:12" ht="30" customHeight="1">
       <c r="A50" s="2">
         <v>48</v>
       </c>
@@ -7123,7 +6501,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="51" customHeight="1" spans="1:12">
+    <row r="51" spans="1:12" ht="30" customHeight="1">
       <c r="A51" s="2">
         <v>49</v>
       </c>
@@ -7158,7 +6536,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="52" customHeight="1" spans="1:12">
+    <row r="52" spans="1:12" ht="30" customHeight="1">
       <c r="A52" s="2">
         <v>50</v>
       </c>
@@ -7193,7 +6571,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="53" customHeight="1" spans="1:12">
+    <row r="53" spans="1:12" ht="30" customHeight="1">
       <c r="A53" s="2">
         <v>51</v>
       </c>
@@ -7228,7 +6606,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="54" customHeight="1" spans="1:12">
+    <row r="54" spans="1:12" ht="30" customHeight="1">
       <c r="A54" s="2">
         <v>52</v>
       </c>
@@ -7263,7 +6641,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="55" ht="70" spans="1:12">
+    <row r="55" spans="1:12" ht="90">
       <c r="A55" s="2">
         <v>53</v>
       </c>
@@ -7295,7 +6673,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="56" ht="70" spans="1:12">
+    <row r="56" spans="1:12" ht="90">
       <c r="A56" s="2">
         <v>54</v>
       </c>
@@ -7327,7 +6705,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="57" ht="56" spans="1:12">
+    <row r="57" spans="1:12" ht="75">
       <c r="A57" s="2">
         <v>55</v>
       </c>
@@ -7359,7 +6737,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="58" ht="56" spans="1:12">
+    <row r="58" spans="1:12" ht="75">
       <c r="A58" s="2">
         <v>56</v>
       </c>
@@ -7391,7 +6769,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="59" ht="56" spans="1:12">
+    <row r="59" spans="1:12" ht="75">
       <c r="A59" s="2">
         <v>57</v>
       </c>
@@ -7423,7 +6801,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="60" ht="56" spans="1:12">
+    <row r="60" spans="1:12" ht="75">
       <c r="A60" s="2">
         <v>58</v>
       </c>
@@ -7455,7 +6833,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="61" ht="56" spans="1:12">
+    <row r="61" spans="1:12" ht="90">
       <c r="A61" s="2">
         <v>59</v>
       </c>
@@ -7487,7 +6865,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="62" ht="56" spans="1:12">
+    <row r="62" spans="1:12" ht="75">
       <c r="A62" s="2">
         <v>60</v>
       </c>
@@ -7519,7 +6897,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="63" ht="56" spans="1:12">
+    <row r="63" spans="1:12" ht="75">
       <c r="A63" s="2">
         <v>61</v>
       </c>
@@ -7551,7 +6929,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="64" ht="56" spans="1:12">
+    <row r="64" spans="1:12" ht="75">
       <c r="A64" s="2">
         <v>62</v>
       </c>
@@ -7583,7 +6961,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="65" ht="56" spans="1:15">
+    <row r="65" spans="1:15" ht="75">
       <c r="A65" s="2">
         <v>63</v>
       </c>
@@ -7615,7 +6993,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="66" ht="14" spans="1:15">
+    <row r="66" spans="1:15" ht="15">
       <c r="A66" s="2">
         <v>64</v>
       </c>
@@ -7647,7 +7025,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="67" ht="14" spans="1:15">
+    <row r="67" spans="1:15" ht="15">
       <c r="A67" s="2">
         <v>65</v>
       </c>
@@ -7679,7 +7057,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="68" ht="14" spans="1:15">
+    <row r="68" spans="1:15" ht="15">
       <c r="A68" s="2">
         <v>66</v>
       </c>
@@ -7711,7 +7089,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="69" ht="14" spans="1:15">
+    <row r="69" spans="1:15" ht="15">
       <c r="A69" s="2">
         <v>67</v>
       </c>
@@ -7743,7 +7121,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="70" ht="14" spans="1:15">
+    <row r="70" spans="1:15" ht="15">
       <c r="A70" s="2">
         <v>68</v>
       </c>
@@ -7775,7 +7153,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="71" ht="14" spans="1:15">
+    <row r="71" spans="1:15" ht="15">
       <c r="A71" s="2">
         <v>69</v>
       </c>
@@ -7807,7 +7185,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="72" ht="14" spans="1:15">
+    <row r="72" spans="1:15" ht="15">
       <c r="A72" s="2">
         <v>70</v>
       </c>
@@ -7839,7 +7217,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="73" ht="14" spans="1:15">
+    <row r="73" spans="1:15" ht="15">
       <c r="A73" s="2">
         <v>71</v>
       </c>
@@ -7868,7 +7246,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="74" ht="42" spans="1:15">
+    <row r="74" spans="1:15" ht="45">
       <c r="A74" s="2">
         <v>72</v>
       </c>
@@ -7909,7 +7287,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="75" ht="14" spans="1:15">
+    <row r="75" spans="1:15" ht="15">
       <c r="A75" s="2">
         <v>73</v>
       </c>
@@ -7935,7 +7313,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="76" customHeight="1" spans="1:15">
+    <row r="76" spans="1:15" ht="30" customHeight="1">
       <c r="A76" s="2">
         <v>74</v>
       </c>
@@ -7964,7 +7342,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="77" customHeight="1" spans="1:15">
+    <row r="77" spans="1:15" ht="30" customHeight="1">
       <c r="A77" s="2">
         <v>75</v>
       </c>
@@ -7999,7 +7377,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="78" customHeight="1" spans="1:15">
+    <row r="78" spans="1:15" ht="30" customHeight="1">
       <c r="A78" s="2">
         <v>76</v>
       </c>
@@ -8034,7 +7412,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="79" customHeight="1" spans="1:15">
+    <row r="79" spans="1:15" ht="30" customHeight="1">
       <c r="A79" s="2">
         <v>77</v>
       </c>
@@ -8069,7 +7447,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="80" customHeight="1" spans="1:15">
+    <row r="80" spans="1:15" ht="30" customHeight="1">
       <c r="A80" s="2">
         <v>78</v>
       </c>
@@ -8104,7 +7482,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="81" customHeight="1" spans="1:14">
+    <row r="81" spans="1:14" ht="30" customHeight="1">
       <c r="A81" s="2">
         <v>79</v>
       </c>
@@ -8139,7 +7517,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="82" customHeight="1" spans="1:14">
+    <row r="82" spans="1:14" ht="30" customHeight="1">
       <c r="A82" s="2">
         <v>80</v>
       </c>
@@ -8168,7 +7546,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="83" customHeight="1" spans="1:14">
+    <row r="83" spans="1:14" ht="30" customHeight="1">
       <c r="A83" s="2">
         <v>81</v>
       </c>
@@ -8194,7 +7572,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="84" customHeight="1" spans="1:14">
+    <row r="84" spans="1:14" ht="30" customHeight="1">
       <c r="A84" s="2">
         <v>82</v>
       </c>
@@ -8222,21 +7600,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="17.2833333333333" customWidth="1"/>
-    <col min="4" max="4" width="20.1416666666667" customWidth="1"/>
-    <col min="5" max="5" width="19.7166666666667" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" customWidth="1"/>
+    <col min="5" max="5" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -8398,21 +7774,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultColWidth="8.71666666666667" defaultRowHeight="14" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.71666666666667" customWidth="1"/>
-    <col min="2" max="2" width="18.7166666666667" customWidth="1"/>
-    <col min="3" max="3" width="11.425" customWidth="1"/>
-    <col min="4" max="4" width="28.85" customWidth="1"/>
-    <col min="5" max="5" width="12.7166666666667" customWidth="1"/>
+    <col min="1" max="1" width="3.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="28.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -8574,22 +7948,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:N10"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.425" customWidth="1"/>
-    <col min="2" max="2" width="15.1416666666667" customWidth="1"/>
-    <col min="3" max="3" width="20.2833333333333" customWidth="1"/>
-    <col min="4" max="5" width="16.85" customWidth="1"/>
-    <col min="7" max="7" width="10.7166666666667" customWidth="1"/>
-    <col min="8" max="8" width="11.2833333333333" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" customWidth="1"/>
+    <col min="3" max="3" width="20.28515625" customWidth="1"/>
+    <col min="4" max="5" width="16.85546875" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -8867,7 +8239,7 @@
         <v>545</v>
       </c>
       <c r="G10" t="s">
-        <v>535</v>
+        <v>0</v>
       </c>
       <c r="H10">
         <v>11</v>
@@ -8887,7 +8259,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>